<commit_message>
reworking the board. Its a prototype not production ready
</commit_message>
<xml_diff>
--- a/Documents/OMNIXIE_sheets.xlsx
+++ b/Documents/OMNIXIE_sheets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21nic\OneDrive\Desktop\NIXIE\OMNIXIE\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E65E5C-CFEB-4DBA-B820-9A9411822778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB799917-C225-4D0E-8E1E-FB18979C06B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="222">
   <si>
     <t>A: ADC, A7 (ADC_IN7)</t>
   </si>
@@ -524,18 +524,6 @@
     <t>C1</t>
   </si>
   <si>
-    <t xml:space="preserve">C0805C105K3RAC </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multilayer Ceramic Capacitors MLCC - SMD/SMT 25V 1uF X7R 0805 10% </t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/ProductDetail/Murata-Electronics/GRM21BR71A106MA73K?qs=QzBtWTOodeUC8P7MOf3tUw%3D%3D</t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/ProductDetail/KEMET/C0805C105K3RAC?qs=ycRbFa0SLRQpHhAu2LUs4g%3D%3D</t>
-  </si>
-  <si>
     <t>C2</t>
   </si>
   <si>
@@ -566,9 +554,6 @@
     <t>R3,R5</t>
   </si>
   <si>
-    <t>4.42m</t>
-  </si>
-  <si>
     <t>15k</t>
   </si>
   <si>
@@ -602,9 +587,6 @@
     <t>Resistor_SMD:R_2010_5025Metric</t>
   </si>
   <si>
-    <t>Resistor_SMD:R_0805_2012Metric</t>
-  </si>
-  <si>
     <t>Resistor_SMD:R_0603_1608Metric</t>
   </si>
   <si>
@@ -662,12 +644,6 @@
     <t xml:space="preserve">Thick Film Resistors - SMD 5.1K ohm 1% </t>
   </si>
   <si>
-    <t xml:space="preserve">RC0402FR-074M42L </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thick Film Resistors General Purpose Chip Resistor 0402, 4.42mOhms, 1%, 1/16W </t>
-  </si>
-  <si>
     <t xml:space="preserve">CRCW04021K50JNEDC </t>
   </si>
   <si>
@@ -680,18 +656,6 @@
     <t xml:space="preserve">RC2010JK-0715KL </t>
   </si>
   <si>
-    <t xml:space="preserve">AC0805DR-071KL </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thick Film Resistors - SMD Automotive Grade Chip Resistor 0805, 1kOhms, 0.5%, 1/8W </t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC0805DR-07100KL </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thick Film Resistors - SMD General Purpose Chip Resistor 0805, 100kOhms, 0.5%, 1/8W </t>
-  </si>
-  <si>
     <t xml:space="preserve">Thick Film Resistors - SMD WRIS-RSKS 47 Ohms 5 % 0.1 W 0402 AEC-Q200 </t>
   </si>
   <si>
@@ -711,6 +675,36 @@
   </si>
   <si>
     <t>J8</t>
+  </si>
+  <si>
+    <t>CL10B105KA8NFNC</t>
+  </si>
+  <si>
+    <t>1 µF ±10% 25V Ceramic Capacitor X7R 0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>RK73H1JTTD1001F</t>
+  </si>
+  <si>
+    <t>1 kOhms ±1% 0.125W, 1/8W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>RC0402FR-07100KL</t>
+  </si>
+  <si>
+    <t>100 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>PA0603FRE570R01L</t>
+  </si>
+  <si>
+    <t>10 mOhms ±1% 0.5W, 1/2W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200, Current Sense, Moisture Resistant Metal Element</t>
+  </si>
+  <si>
+    <t>10m</t>
+  </si>
+  <si>
+    <t>Capacitor_SMD:C_0603_1608Metric</t>
   </si>
 </sst>
 </file>
@@ -1489,7 +1483,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="187">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1637,65 +1631,12 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1711,7 +1652,7 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1724,45 +1665,30 @@
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1812,7 +1738,7 @@
     <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1845,13 +1771,12 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1872,7 +1797,7 @@
     <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1881,14 +1806,13 @@
     <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="15" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1938,11 +1862,68 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2462,7 +2443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10C7034E-99F6-4C64-9A78-788C06E81851}">
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -2471,7 +2452,7 @@
     <col min="4" max="4" width="16.28515625" customWidth="1"/>
     <col min="5" max="5" width="9.85546875" customWidth="1"/>
     <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="90.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="121.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="59.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -2479,856 +2460,745 @@
     <col min="12" max="12" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
         <v>142</v>
       </c>
       <c r="B1" s="40">
         <v>1</v>
       </c>
-      <c r="C1" s="66" t="s">
+      <c r="C1" s="169" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="68"/>
+      <c r="D1" s="170"/>
+      <c r="E1" s="170"/>
+      <c r="F1" s="170"/>
+      <c r="G1" s="170"/>
+      <c r="H1" s="170"/>
+      <c r="I1" s="170"/>
+      <c r="J1" s="170"/>
+      <c r="K1" s="171"/>
       <c r="L1" s="36"/>
       <c r="M1" s="36"/>
     </row>
-    <row r="2" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="41" t="s">
         <v>143</v>
       </c>
       <c r="B2" s="40">
         <v>1</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="71"/>
+      <c r="C2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
+      <c r="G2" s="173"/>
+      <c r="H2" s="173"/>
+      <c r="I2" s="173"/>
+      <c r="J2" s="173"/>
+      <c r="K2" s="174"/>
       <c r="L2" s="36"/>
       <c r="M2" s="36"/>
     </row>
-    <row r="3" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41" t="s">
         <v>144</v>
       </c>
       <c r="B3" s="40">
         <v>1</v>
       </c>
-      <c r="C3" s="60" t="s">
+      <c r="C3" s="163" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
+      <c r="D3" s="164"/>
+      <c r="E3" s="164"/>
+      <c r="F3" s="164"/>
+      <c r="G3" s="164"/>
+      <c r="H3" s="164"/>
+      <c r="I3" s="164"/>
+      <c r="J3" s="164"/>
+      <c r="K3" s="165"/>
       <c r="L3" s="36"/>
       <c r="M3" s="36"/>
     </row>
-    <row r="4" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="171" t="s">
+    <row r="4" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="147" t="s">
         <v>140</v>
       </c>
-      <c r="B4" s="172">
+      <c r="B4" s="148">
         <v>46009</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="65"/>
+      <c r="C4" s="166"/>
+      <c r="D4" s="167"/>
+      <c r="E4" s="167"/>
+      <c r="F4" s="167"/>
+      <c r="G4" s="167"/>
+      <c r="H4" s="167"/>
+      <c r="I4" s="167"/>
+      <c r="J4" s="167"/>
+      <c r="K4" s="168"/>
       <c r="L4" s="36"/>
       <c r="M4" s="36"/>
     </row>
-    <row r="5" spans="1:18" s="145" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="181" t="s">
+    <row r="5" spans="1:13" s="122" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="157" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="182" t="s">
+      <c r="B5" s="158" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="182" t="s">
+      <c r="C5" s="158" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="182" t="s">
+      <c r="D5" s="158" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="182" t="s">
-        <v>169</v>
-      </c>
-      <c r="F5" s="182" t="s">
+      <c r="E5" s="158" t="s">
+        <v>165</v>
+      </c>
+      <c r="F5" s="158" t="s">
         <v>145</v>
       </c>
-      <c r="G5" s="183" t="s">
+      <c r="G5" s="159" t="s">
         <v>95</v>
       </c>
-      <c r="H5" s="182" t="s">
+      <c r="H5" s="158" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="182" t="s">
+      <c r="I5" s="158" t="s">
         <v>136</v>
       </c>
-      <c r="J5" s="182" t="s">
+      <c r="J5" s="158" t="s">
         <v>137</v>
       </c>
-      <c r="K5" s="184" t="s">
+      <c r="K5" s="160" t="s">
         <v>138</v>
       </c>
-      <c r="L5" s="143"/>
-      <c r="M5" s="143"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="173" t="s">
+      <c r="L5" s="121"/>
+      <c r="M5" s="121"/>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="149" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="174">
+      <c r="B6" s="150">
         <v>1</v>
       </c>
-      <c r="C6" s="174" t="s">
+      <c r="C6" s="150" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="175" t="s">
-        <v>192</v>
-      </c>
-      <c r="E6" s="176" t="s">
-        <v>170</v>
-      </c>
-      <c r="F6" s="177"/>
-      <c r="G6" s="178" t="s">
+      <c r="D6" s="151" t="s">
+        <v>186</v>
+      </c>
+      <c r="E6" s="152" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="153"/>
+      <c r="G6" s="154" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="179"/>
-      <c r="I6" s="179"/>
-      <c r="J6" s="179"/>
-      <c r="K6" s="180"/>
+      <c r="H6" s="155"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="155"/>
+      <c r="K6" s="156"/>
       <c r="L6" s="36"/>
       <c r="M6" s="36"/>
-      <c r="N6" s="75"/>
-      <c r="O6" s="75"/>
-      <c r="P6" s="75"/>
-      <c r="Q6" s="75"/>
-      <c r="R6" s="75"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="119"/>
-      <c r="B7" s="120">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="97"/>
+      <c r="B7" s="98">
         <v>1</v>
       </c>
-      <c r="C7" s="120" t="s">
+      <c r="C7" s="98" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="121" t="s">
-        <v>193</v>
-      </c>
-      <c r="E7" s="122" t="s">
-        <v>170</v>
-      </c>
-      <c r="F7" s="123"/>
-      <c r="G7" s="124" t="s">
+      <c r="D7" s="99" t="s">
+        <v>187</v>
+      </c>
+      <c r="E7" s="100" t="s">
+        <v>166</v>
+      </c>
+      <c r="F7" s="101"/>
+      <c r="G7" s="102" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="125"/>
-      <c r="I7" s="125"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="126"/>
+      <c r="H7" s="103"/>
+      <c r="I7" s="103"/>
+      <c r="J7" s="103"/>
+      <c r="K7" s="104"/>
       <c r="L7" s="36"/>
       <c r="M7" s="36"/>
-      <c r="N7" s="75"/>
-      <c r="O7" s="75"/>
-      <c r="P7" s="75"/>
-      <c r="Q7" s="75"/>
-      <c r="R7" s="75"/>
-    </row>
-    <row r="8" spans="1:18" s="145" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="135"/>
-      <c r="B8" s="136">
+    </row>
+    <row r="8" spans="1:13" s="122" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="113"/>
+      <c r="B8" s="114">
         <v>1</v>
       </c>
-      <c r="C8" s="136" t="s">
+      <c r="C8" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="137" t="s">
-        <v>194</v>
-      </c>
-      <c r="E8" s="138" t="s">
-        <v>170</v>
-      </c>
-      <c r="F8" s="139"/>
-      <c r="G8" s="140" t="s">
+      <c r="D8" s="115" t="s">
+        <v>188</v>
+      </c>
+      <c r="E8" s="116" t="s">
+        <v>166</v>
+      </c>
+      <c r="F8" s="117"/>
+      <c r="G8" s="118" t="s">
         <v>104</v>
       </c>
-      <c r="H8" s="141"/>
-      <c r="I8" s="141"/>
-      <c r="J8" s="141"/>
-      <c r="K8" s="142"/>
-      <c r="L8" s="143"/>
-      <c r="M8" s="143"/>
-      <c r="N8" s="144"/>
-      <c r="O8" s="144"/>
-      <c r="P8" s="144"/>
-      <c r="Q8" s="144"/>
-      <c r="R8" s="144"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="127" t="s">
+      <c r="H8" s="119"/>
+      <c r="I8" s="119"/>
+      <c r="J8" s="119"/>
+      <c r="K8" s="120"/>
+      <c r="L8" s="121"/>
+      <c r="M8" s="121"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="105" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="128">
+      <c r="B9" s="106">
         <v>1</v>
       </c>
-      <c r="C9" s="186" t="s">
-        <v>220</v>
-      </c>
-      <c r="D9" s="129" t="s">
-        <v>195</v>
-      </c>
-      <c r="E9" s="130" t="s">
-        <v>170</v>
-      </c>
-      <c r="F9" s="131"/>
-      <c r="G9" s="132" t="s">
+      <c r="C9" s="162" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="107" t="s">
+        <v>189</v>
+      </c>
+      <c r="E9" s="108" t="s">
+        <v>166</v>
+      </c>
+      <c r="F9" s="109"/>
+      <c r="G9" s="110" t="s">
         <v>103</v>
       </c>
-      <c r="H9" s="133"/>
-      <c r="I9" s="133"/>
-      <c r="J9" s="133"/>
-      <c r="K9" s="134"/>
+      <c r="H9" s="111"/>
+      <c r="I9" s="111"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="112"/>
       <c r="L9" s="36"/>
       <c r="M9" s="36"/>
-      <c r="N9" s="75"/>
-      <c r="O9" s="75"/>
-      <c r="P9" s="75"/>
-      <c r="Q9" s="75"/>
-      <c r="R9" s="75"/>
-    </row>
-    <row r="10" spans="1:18" s="73" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="106"/>
-      <c r="B10" s="77">
+    </row>
+    <row r="10" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="84"/>
+      <c r="B10" s="62">
         <v>2</v>
       </c>
-      <c r="C10" s="77" t="s">
-        <v>170</v>
-      </c>
-      <c r="D10" s="78" t="s">
-        <v>202</v>
-      </c>
-      <c r="E10" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F10" s="80" t="s">
-        <v>204</v>
-      </c>
-      <c r="G10" s="81" t="s">
-        <v>203</v>
-      </c>
-      <c r="H10" s="82"/>
-      <c r="I10" s="82"/>
-      <c r="J10" s="82"/>
-      <c r="K10" s="107"/>
-      <c r="L10" s="74"/>
-      <c r="M10" s="74"/>
-      <c r="N10" s="76"/>
-      <c r="O10" s="76"/>
-      <c r="P10" s="76"/>
-      <c r="Q10" s="76"/>
-      <c r="R10" s="76"/>
-    </row>
-    <row r="11" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="108"/>
-      <c r="B11" s="77">
+      <c r="C10" s="62" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" s="63" t="s">
+        <v>196</v>
+      </c>
+      <c r="E10" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F10" s="65" t="s">
+        <v>198</v>
+      </c>
+      <c r="G10" s="66" t="s">
+        <v>197</v>
+      </c>
+      <c r="H10" s="67"/>
+      <c r="I10" s="67"/>
+      <c r="J10" s="67"/>
+      <c r="K10" s="85"/>
+      <c r="L10" s="61"/>
+      <c r="M10" s="61"/>
+    </row>
+    <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="86"/>
+      <c r="B11" s="62">
         <v>1</v>
       </c>
-      <c r="C11" s="77">
+      <c r="C11" s="62">
         <v>5005</v>
       </c>
-      <c r="D11" s="78" t="s">
-        <v>197</v>
-      </c>
-      <c r="E11" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F11" s="80"/>
-      <c r="G11" s="81" t="s">
+      <c r="D11" s="63" t="s">
+        <v>191</v>
+      </c>
+      <c r="E11" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F11" s="65"/>
+      <c r="G11" s="66" t="s">
         <v>108</v>
       </c>
-      <c r="H11" s="82"/>
-      <c r="I11" s="82"/>
-      <c r="J11" s="82"/>
-      <c r="K11" s="107"/>
-      <c r="L11" s="75"/>
-      <c r="M11" s="75"/>
-      <c r="N11" s="75"/>
-      <c r="O11" s="75"/>
-      <c r="P11" s="75"/>
-      <c r="Q11" s="75"/>
-      <c r="R11" s="75"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="108"/>
-      <c r="B12" s="77">
+      <c r="H11" s="67"/>
+      <c r="I11" s="67"/>
+      <c r="J11" s="67"/>
+      <c r="K11" s="85"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="86"/>
+      <c r="B12" s="62">
         <v>2</v>
       </c>
-      <c r="C12" s="77" t="s">
+      <c r="C12" s="62" t="s">
         <v>101</v>
       </c>
-      <c r="D12" s="83" t="s">
-        <v>196</v>
-      </c>
-      <c r="E12" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F12" s="80"/>
-      <c r="G12" s="81" t="s">
+      <c r="D12" s="68" t="s">
+        <v>190</v>
+      </c>
+      <c r="E12" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F12" s="65"/>
+      <c r="G12" s="66" t="s">
         <v>102</v>
       </c>
-      <c r="H12" s="82"/>
-      <c r="I12" s="82"/>
-      <c r="J12" s="82"/>
-      <c r="K12" s="107"/>
+      <c r="H12" s="67"/>
+      <c r="I12" s="67"/>
+      <c r="J12" s="67"/>
+      <c r="K12" s="85"/>
       <c r="L12" s="36"/>
       <c r="M12" s="36"/>
-      <c r="N12" s="75"/>
-      <c r="O12" s="75"/>
-      <c r="P12" s="75"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="75"/>
-    </row>
-    <row r="13" spans="1:18" s="73" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="108"/>
-      <c r="B13" s="77">
+    </row>
+    <row r="13" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="86"/>
+      <c r="B13" s="62">
         <v>1</v>
       </c>
-      <c r="C13" s="77" t="s">
+      <c r="C13" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="83" t="s">
-        <v>223</v>
-      </c>
-      <c r="E13" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F13" s="80"/>
-      <c r="G13" s="81" t="s">
-        <v>221</v>
-      </c>
-      <c r="H13" s="82"/>
-      <c r="I13" s="82"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="107"/>
-      <c r="L13" s="74"/>
-      <c r="M13" s="74"/>
-      <c r="N13" s="76"/>
-      <c r="O13" s="76"/>
-      <c r="P13" s="76"/>
-      <c r="Q13" s="76"/>
-      <c r="R13" s="76"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="108"/>
-      <c r="B14" s="77">
+      <c r="D13" s="68" t="s">
+        <v>211</v>
+      </c>
+      <c r="E13" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F13" s="65"/>
+      <c r="G13" s="66" t="s">
+        <v>209</v>
+      </c>
+      <c r="H13" s="67"/>
+      <c r="I13" s="67"/>
+      <c r="J13" s="67"/>
+      <c r="K13" s="85"/>
+      <c r="L13" s="61"/>
+      <c r="M13" s="61"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="86"/>
+      <c r="B14" s="62">
         <v>1</v>
       </c>
-      <c r="C14" s="77" t="s">
+      <c r="C14" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="D14" s="84" t="s">
-        <v>199</v>
-      </c>
-      <c r="E14" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F14" s="80"/>
-      <c r="G14" s="81" t="s">
+      <c r="D14" s="69" t="s">
+        <v>193</v>
+      </c>
+      <c r="E14" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F14" s="65"/>
+      <c r="G14" s="66" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="82"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="82"/>
-      <c r="K14" s="107"/>
+      <c r="H14" s="67"/>
+      <c r="I14" s="67"/>
+      <c r="J14" s="67"/>
+      <c r="K14" s="85"/>
       <c r="L14" s="36"/>
       <c r="M14" s="36"/>
-      <c r="N14" s="75"/>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-    </row>
-    <row r="15" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="108"/>
-      <c r="B15" s="77">
+    </row>
+    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="86"/>
+      <c r="B15" s="62">
         <v>12</v>
       </c>
-      <c r="C15" s="77" t="s">
+      <c r="C15" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="84" t="s">
-        <v>198</v>
-      </c>
-      <c r="E15" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F15" s="80"/>
-      <c r="G15" s="81" t="s">
+      <c r="D15" s="69" t="s">
+        <v>192</v>
+      </c>
+      <c r="E15" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F15" s="65"/>
+      <c r="G15" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="H15" s="82"/>
-      <c r="I15" s="82"/>
-      <c r="J15" s="82"/>
-      <c r="K15" s="107"/>
+      <c r="H15" s="67"/>
+      <c r="I15" s="67"/>
+      <c r="J15" s="67"/>
+      <c r="K15" s="85"/>
       <c r="L15" s="36"/>
       <c r="M15" s="36"/>
-      <c r="N15" s="75"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="75"/>
-      <c r="R15" s="75"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="146"/>
-      <c r="B16" s="147">
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="123"/>
+      <c r="B16" s="124">
         <v>1</v>
       </c>
-      <c r="C16" s="147" t="s">
+      <c r="C16" s="124" t="s">
         <v>113</v>
       </c>
-      <c r="D16" s="148" t="s">
-        <v>200</v>
-      </c>
-      <c r="E16" s="149" t="s">
-        <v>170</v>
-      </c>
-      <c r="F16" s="150"/>
-      <c r="G16" s="151" t="s">
+      <c r="D16" s="125" t="s">
+        <v>194</v>
+      </c>
+      <c r="E16" s="126" t="s">
+        <v>166</v>
+      </c>
+      <c r="F16" s="127"/>
+      <c r="G16" s="128" t="s">
         <v>123</v>
       </c>
-      <c r="H16" s="152"/>
-      <c r="I16" s="152"/>
-      <c r="J16" s="152"/>
-      <c r="K16" s="153"/>
+      <c r="H16" s="129"/>
+      <c r="I16" s="129"/>
+      <c r="J16" s="129"/>
+      <c r="K16" s="130"/>
       <c r="L16" s="36"/>
       <c r="M16" s="36"/>
-      <c r="N16" s="75"/>
-      <c r="O16" s="75"/>
-      <c r="P16" s="75"/>
-      <c r="Q16" s="75"/>
-      <c r="R16" s="75"/>
-    </row>
-    <row r="17" spans="1:18" s="145" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="163"/>
-      <c r="B17" s="164">
+    </row>
+    <row r="17" spans="1:13" s="122" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="139"/>
+      <c r="B17" s="140">
         <v>1</v>
       </c>
-      <c r="C17" s="164" t="s">
+      <c r="C17" s="140" t="s">
         <v>121</v>
       </c>
-      <c r="D17" s="165" t="s">
-        <v>201</v>
-      </c>
-      <c r="E17" s="166" t="s">
-        <v>170</v>
-      </c>
-      <c r="F17" s="167"/>
-      <c r="G17" s="168" t="s">
+      <c r="D17" s="141" t="s">
+        <v>195</v>
+      </c>
+      <c r="E17" s="142" t="s">
+        <v>166</v>
+      </c>
+      <c r="F17" s="143"/>
+      <c r="G17" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="H17" s="169"/>
-      <c r="I17" s="169"/>
-      <c r="J17" s="169"/>
-      <c r="K17" s="170"/>
-      <c r="L17" s="143"/>
-      <c r="M17" s="143"/>
-      <c r="N17" s="144"/>
-      <c r="O17" s="144"/>
-      <c r="P17" s="144"/>
-      <c r="Q17" s="144"/>
-      <c r="R17" s="144"/>
-    </row>
-    <row r="18" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="154" t="s">
-        <v>191</v>
-      </c>
-      <c r="B18" s="155">
+      <c r="H17" s="145"/>
+      <c r="I17" s="145"/>
+      <c r="J17" s="145"/>
+      <c r="K17" s="146"/>
+      <c r="L17" s="121"/>
+      <c r="M17" s="121"/>
+    </row>
+    <row r="18" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="131" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="132">
         <v>1</v>
       </c>
-      <c r="C18" s="155" t="s">
+      <c r="C18" s="132" t="s">
         <v>158</v>
       </c>
-      <c r="D18" s="156" t="s">
+      <c r="D18" s="133" t="s">
         <v>160</v>
       </c>
-      <c r="E18" s="157" t="s">
-        <v>171</v>
-      </c>
-      <c r="F18" s="158"/>
-      <c r="G18" s="159" t="s">
+      <c r="E18" s="134" t="s">
+        <v>167</v>
+      </c>
+      <c r="F18" s="135"/>
+      <c r="G18" s="136" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="160" t="s">
-        <v>189</v>
-      </c>
-      <c r="I18" s="161"/>
-      <c r="J18" s="161"/>
-      <c r="K18" s="162" t="s">
-        <v>163</v>
-      </c>
+      <c r="H18" s="176" t="s">
+        <v>183</v>
+      </c>
+      <c r="I18" s="137"/>
+      <c r="J18" s="137"/>
+      <c r="K18" s="138"/>
       <c r="L18" s="36"/>
       <c r="M18" s="36"/>
-      <c r="N18" s="75"/>
-      <c r="O18" s="75"/>
-      <c r="P18" s="75"/>
-      <c r="Q18" s="75"/>
-      <c r="R18" s="75"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="109"/>
-      <c r="B19" s="86">
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="87"/>
+      <c r="B19" s="71">
         <v>1</v>
       </c>
-      <c r="C19" s="87" t="s">
-        <v>218</v>
-      </c>
-      <c r="D19" s="88" t="s">
-        <v>165</v>
-      </c>
-      <c r="E19" s="89" t="s">
-        <v>172</v>
-      </c>
-      <c r="F19" s="90"/>
-      <c r="G19" s="87" t="s">
-        <v>219</v>
-      </c>
-      <c r="H19" s="91" t="s">
-        <v>190</v>
-      </c>
-      <c r="I19" s="85"/>
-      <c r="J19" s="85"/>
-      <c r="K19" s="110" t="s">
-        <v>164</v>
-      </c>
+      <c r="C19" s="71" t="s">
+        <v>206</v>
+      </c>
+      <c r="D19" s="73" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="74" t="s">
+        <v>168</v>
+      </c>
+      <c r="F19" s="75"/>
+      <c r="G19" s="72" t="s">
+        <v>207</v>
+      </c>
+      <c r="H19" s="177" t="s">
+        <v>184</v>
+      </c>
+      <c r="I19" s="70"/>
+      <c r="J19" s="70"/>
+      <c r="K19" s="88"/>
       <c r="L19" s="36"/>
       <c r="M19" s="36"/>
-      <c r="N19" s="75"/>
-      <c r="O19" s="75"/>
-      <c r="P19" s="75"/>
-      <c r="Q19" s="75"/>
-      <c r="R19" s="75"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="109"/>
-      <c r="B20" s="86">
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="87"/>
+      <c r="B20" s="71">
         <v>1</v>
       </c>
-      <c r="C20" s="86" t="s">
-        <v>161</v>
-      </c>
-      <c r="D20" s="88" t="s">
-        <v>166</v>
-      </c>
-      <c r="E20" s="89" t="s">
-        <v>173</v>
-      </c>
-      <c r="F20" s="90"/>
-      <c r="G20" s="92" t="s">
+      <c r="C20" s="71" t="s">
+        <v>212</v>
+      </c>
+      <c r="D20" s="73" t="s">
         <v>162</v>
       </c>
-      <c r="H20" s="91" t="s">
-        <v>189</v>
-      </c>
-      <c r="I20" s="85"/>
-      <c r="J20" s="85"/>
-      <c r="K20" s="110"/>
+      <c r="E20" s="74" t="s">
+        <v>169</v>
+      </c>
+      <c r="F20" s="75"/>
+      <c r="G20" s="76" t="s">
+        <v>213</v>
+      </c>
+      <c r="H20" s="177" t="s">
+        <v>221</v>
+      </c>
+      <c r="I20" s="70"/>
+      <c r="J20" s="70"/>
+      <c r="K20" s="88"/>
       <c r="L20" s="36"/>
       <c r="M20" s="36"/>
-      <c r="N20" s="75"/>
-      <c r="O20" s="75"/>
-      <c r="P20" s="75"/>
-      <c r="Q20" s="75"/>
-      <c r="R20" s="75"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="109"/>
-      <c r="B21" s="93">
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="87"/>
+      <c r="B21" s="77">
         <v>2</v>
       </c>
-      <c r="C21" s="93" t="s">
-        <v>207</v>
-      </c>
-      <c r="D21" s="94" t="s">
-        <v>174</v>
-      </c>
-      <c r="E21" s="89" t="s">
-        <v>175</v>
-      </c>
-      <c r="F21" s="95"/>
-      <c r="G21" s="96" t="s">
-        <v>208</v>
-      </c>
-      <c r="H21" s="97" t="s">
-        <v>185</v>
-      </c>
-      <c r="I21" s="85"/>
-      <c r="J21" s="85"/>
-      <c r="K21" s="110"/>
+      <c r="C21" s="77" t="s">
+        <v>218</v>
+      </c>
+      <c r="D21" s="78" t="s">
+        <v>170</v>
+      </c>
+      <c r="E21" s="74" t="s">
+        <v>220</v>
+      </c>
+      <c r="F21" s="79"/>
+      <c r="G21" s="80" t="s">
+        <v>219</v>
+      </c>
+      <c r="H21" s="177" t="s">
+        <v>182</v>
+      </c>
+      <c r="I21" s="70"/>
+      <c r="J21" s="70"/>
+      <c r="K21" s="88"/>
       <c r="L21" s="36"/>
       <c r="M21" s="36"/>
-      <c r="N21" s="75"/>
-      <c r="O21" s="75"/>
-      <c r="P21" s="75"/>
-      <c r="Q21" s="75"/>
-      <c r="R21" s="75"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="109"/>
-      <c r="B22" s="93">
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="87"/>
+      <c r="B22" s="77">
         <v>1</v>
       </c>
-      <c r="C22" s="86" t="s">
-        <v>212</v>
-      </c>
-      <c r="D22" s="94" t="s">
-        <v>167</v>
-      </c>
-      <c r="E22" s="89" t="s">
-        <v>176</v>
-      </c>
-      <c r="F22" s="90"/>
-      <c r="G22" s="92" t="s">
-        <v>211</v>
-      </c>
-      <c r="H22" s="97" t="s">
-        <v>186</v>
-      </c>
-      <c r="I22" s="85"/>
-      <c r="J22" s="85"/>
-      <c r="K22" s="110"/>
+      <c r="C22" s="71" t="s">
+        <v>204</v>
+      </c>
+      <c r="D22" s="78" t="s">
+        <v>163</v>
+      </c>
+      <c r="E22" s="74" t="s">
+        <v>171</v>
+      </c>
+      <c r="F22" s="75"/>
+      <c r="G22" s="76" t="s">
+        <v>203</v>
+      </c>
+      <c r="H22" s="177" t="s">
+        <v>181</v>
+      </c>
+      <c r="I22" s="70"/>
+      <c r="J22" s="70"/>
+      <c r="K22" s="88"/>
       <c r="L22" s="36"/>
       <c r="M22" s="36"/>
-      <c r="N22" s="75"/>
-      <c r="O22" s="75"/>
-      <c r="P22" s="75"/>
-      <c r="Q22" s="75"/>
-      <c r="R22" s="75"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="109"/>
-      <c r="B23" s="93">
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="87"/>
+      <c r="B23" s="77">
         <v>1</v>
       </c>
-      <c r="C23" s="86" t="s">
-        <v>215</v>
-      </c>
-      <c r="D23" s="94" t="s">
-        <v>168</v>
-      </c>
-      <c r="E23" s="89" t="s">
-        <v>177</v>
-      </c>
-      <c r="F23" s="90"/>
-      <c r="G23" s="92" t="s">
+      <c r="C23" s="71" t="s">
         <v>216</v>
       </c>
-      <c r="H23" s="97" t="s">
-        <v>187</v>
-      </c>
-      <c r="I23" s="85"/>
-      <c r="J23" s="85"/>
-      <c r="K23" s="110"/>
+      <c r="D23" s="78" t="s">
+        <v>164</v>
+      </c>
+      <c r="E23" s="74" t="s">
+        <v>172</v>
+      </c>
+      <c r="F23" s="75"/>
+      <c r="G23" s="76" t="s">
+        <v>217</v>
+      </c>
+      <c r="H23" s="177" t="s">
+        <v>180</v>
+      </c>
+      <c r="I23" s="70"/>
+      <c r="J23" s="70"/>
+      <c r="K23" s="88"/>
       <c r="L23" s="36"/>
       <c r="M23" s="36"/>
-      <c r="N23" s="75"/>
-      <c r="O23" s="75"/>
-      <c r="P23" s="75"/>
-      <c r="Q23" s="75"/>
-      <c r="R23" s="75"/>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="109"/>
-      <c r="B24" s="93">
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="87"/>
+      <c r="B24" s="77">
         <v>2</v>
       </c>
-      <c r="C24" s="185">
+      <c r="C24" s="161">
         <v>560112110017</v>
       </c>
-      <c r="D24" s="94" t="s">
-        <v>178</v>
-      </c>
-      <c r="E24" s="89">
+      <c r="D24" s="78" t="s">
+        <v>173</v>
+      </c>
+      <c r="E24" s="74">
         <v>47</v>
       </c>
-      <c r="F24" s="95"/>
-      <c r="G24" s="96" t="s">
-        <v>217</v>
-      </c>
-      <c r="H24" s="97" t="s">
-        <v>185</v>
-      </c>
-      <c r="I24" s="85"/>
-      <c r="J24" s="85"/>
-      <c r="K24" s="110"/>
+      <c r="F24" s="79"/>
+      <c r="G24" s="80" t="s">
+        <v>205</v>
+      </c>
+      <c r="H24" s="177" t="s">
+        <v>180</v>
+      </c>
+      <c r="I24" s="70"/>
+      <c r="J24" s="70"/>
+      <c r="K24" s="88"/>
       <c r="L24" s="36"/>
       <c r="M24" s="36"/>
-      <c r="N24" s="75"/>
-      <c r="O24" s="75"/>
-      <c r="P24" s="75"/>
-      <c r="Q24" s="75"/>
-      <c r="R24" s="75"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25" s="109"/>
-      <c r="B25" s="93">
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="87"/>
+      <c r="B25" s="77">
         <v>2</v>
       </c>
-      <c r="C25" s="93" t="s">
-        <v>213</v>
-      </c>
-      <c r="D25" s="94" t="s">
-        <v>179</v>
-      </c>
-      <c r="E25" s="89" t="s">
-        <v>180</v>
-      </c>
-      <c r="F25" s="95"/>
-      <c r="G25" s="96" t="s">
+      <c r="C25" s="77" t="s">
         <v>214</v>
       </c>
-      <c r="H25" s="97" t="s">
-        <v>187</v>
-      </c>
-      <c r="I25" s="85"/>
-      <c r="J25" s="85"/>
-      <c r="K25" s="110"/>
+      <c r="D25" s="78" t="s">
+        <v>174</v>
+      </c>
+      <c r="E25" s="74" t="s">
+        <v>175</v>
+      </c>
+      <c r="F25" s="79"/>
+      <c r="G25" s="80" t="s">
+        <v>215</v>
+      </c>
+      <c r="H25" s="177" t="s">
+        <v>182</v>
+      </c>
+      <c r="I25" s="70"/>
+      <c r="J25" s="70"/>
+      <c r="K25" s="88"/>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
-      <c r="N25" s="75"/>
-      <c r="O25" s="75"/>
-      <c r="P25" s="75"/>
-      <c r="Q25" s="75"/>
-      <c r="R25" s="75"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="109"/>
-      <c r="B26" s="93">
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="87"/>
+      <c r="B26" s="77">
         <v>2</v>
       </c>
-      <c r="C26" s="93" t="s">
-        <v>205</v>
-      </c>
-      <c r="D26" s="94" t="s">
-        <v>181</v>
-      </c>
-      <c r="E26" s="89" t="s">
+      <c r="C26" s="77" t="s">
+        <v>199</v>
+      </c>
+      <c r="D26" s="78" t="s">
+        <v>176</v>
+      </c>
+      <c r="E26" s="74" t="s">
+        <v>177</v>
+      </c>
+      <c r="F26" s="79"/>
+      <c r="G26" s="81" t="s">
+        <v>200</v>
+      </c>
+      <c r="H26" s="177" t="s">
         <v>182</v>
       </c>
-      <c r="F26" s="95"/>
-      <c r="G26" s="98" t="s">
-        <v>206</v>
-      </c>
-      <c r="H26" s="97" t="s">
-        <v>188</v>
-      </c>
-      <c r="I26" s="85"/>
-      <c r="J26" s="85"/>
-      <c r="K26" s="110"/>
+      <c r="I26" s="70"/>
+      <c r="J26" s="70"/>
+      <c r="K26" s="88"/>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
-      <c r="N26" s="75"/>
-      <c r="O26" s="75"/>
-      <c r="P26" s="75"/>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="75"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="109"/>
-      <c r="B27" s="99">
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="87"/>
+      <c r="B27" s="77">
         <v>1</v>
       </c>
-      <c r="C27" s="99" t="s">
-        <v>209</v>
-      </c>
-      <c r="D27" s="101" t="s">
-        <v>183</v>
-      </c>
-      <c r="E27" s="102" t="s">
-        <v>184</v>
-      </c>
-      <c r="F27" s="95"/>
-      <c r="G27" s="100" t="s">
-        <v>210</v>
-      </c>
-      <c r="H27" s="103" t="s">
-        <v>185</v>
-      </c>
-      <c r="I27" s="85"/>
-      <c r="J27" s="85"/>
-      <c r="K27" s="110"/>
+      <c r="C27" s="77" t="s">
+        <v>201</v>
+      </c>
+      <c r="D27" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E27" s="74" t="s">
+        <v>179</v>
+      </c>
+      <c r="F27" s="79"/>
+      <c r="G27" s="81" t="s">
+        <v>202</v>
+      </c>
+      <c r="H27" s="177" t="s">
+        <v>180</v>
+      </c>
+      <c r="I27" s="70"/>
+      <c r="J27" s="70"/>
+      <c r="K27" s="88"/>
       <c r="L27" s="36"/>
       <c r="M27" s="36"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="109"/>
-      <c r="B28" s="104"/>
-      <c r="C28" s="87"/>
-      <c r="D28" s="105"/>
-      <c r="E28" s="85"/>
-      <c r="F28" s="90"/>
-      <c r="G28" s="87"/>
-      <c r="H28" s="85"/>
-      <c r="I28" s="85"/>
-      <c r="J28" s="85"/>
-      <c r="K28" s="110"/>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="87"/>
+      <c r="B28" s="82"/>
+      <c r="C28" s="72"/>
+      <c r="D28" s="83"/>
+      <c r="E28" s="70"/>
+      <c r="F28" s="75"/>
+      <c r="G28" s="72"/>
+      <c r="H28" s="70"/>
+      <c r="I28" s="70"/>
+      <c r="J28" s="70"/>
+      <c r="K28" s="88"/>
       <c r="L28" s="36"/>
       <c r="M28" s="36"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="109"/>
-      <c r="B29" s="104"/>
-      <c r="C29" s="85"/>
-      <c r="D29" s="105"/>
-      <c r="E29" s="85"/>
-      <c r="F29" s="90"/>
-      <c r="G29" s="87"/>
-      <c r="H29" s="85"/>
-      <c r="I29" s="85"/>
-      <c r="J29" s="85"/>
-      <c r="K29" s="110"/>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="87"/>
+      <c r="B29" s="82"/>
+      <c r="C29" s="70"/>
+      <c r="D29" s="83"/>
+      <c r="E29" s="70"/>
+      <c r="F29" s="75"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="70"/>
+      <c r="I29" s="70"/>
+      <c r="J29" s="70"/>
+      <c r="K29" s="88"/>
       <c r="L29" s="36"/>
       <c r="M29" s="36"/>
     </row>
-    <row r="30" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="111"/>
-      <c r="B30" s="112"/>
-      <c r="C30" s="113"/>
-      <c r="D30" s="114"/>
-      <c r="E30" s="115"/>
-      <c r="F30" s="116"/>
-      <c r="G30" s="117"/>
-      <c r="H30" s="115"/>
-      <c r="I30" s="115"/>
-      <c r="J30" s="115"/>
-      <c r="K30" s="118"/>
+    <row r="30" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="89"/>
+      <c r="B30" s="90"/>
+      <c r="C30" s="91"/>
+      <c r="D30" s="92"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="94"/>
+      <c r="G30" s="95"/>
+      <c r="H30" s="93"/>
+      <c r="I30" s="93"/>
+      <c r="J30" s="93"/>
+      <c r="K30" s="96"/>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="33"/>
       <c r="B31" s="33"/>
       <c r="C31" s="33"/>
@@ -3343,7 +3213,7 @@
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="33"/>
       <c r="B32" s="33"/>
       <c r="C32" s="33"/>
@@ -3358,33 +3228,28 @@
       <c r="L32" s="36"/>
       <c r="M32" s="36"/>
     </row>
-    <row r="33" spans="1:18" s="73" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="108"/>
-      <c r="B33" s="77">
+    <row r="33" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="86"/>
+      <c r="B33" s="62">
         <v>1</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="D33" s="83"/>
-      <c r="E33" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="F33" s="80"/>
-      <c r="G33" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="H33" s="82"/>
-      <c r="I33" s="82"/>
-      <c r="J33" s="82"/>
-      <c r="K33" s="107"/>
-      <c r="L33" s="74"/>
-      <c r="M33" s="74"/>
-      <c r="N33" s="76"/>
-      <c r="O33" s="76"/>
-      <c r="P33" s="76"/>
-      <c r="Q33" s="76"/>
-      <c r="R33" s="76"/>
+      <c r="D33" s="68"/>
+      <c r="E33" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F33" s="65"/>
+      <c r="G33" s="66" t="s">
+        <v>210</v>
+      </c>
+      <c r="H33" s="67"/>
+      <c r="I33" s="67"/>
+      <c r="J33" s="67"/>
+      <c r="K33" s="85"/>
+      <c r="L33" s="61"/>
+      <c r="M33" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3418,14 +3283,14 @@
       <c r="E2" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="72" t="s">
+      <c r="F2" s="175" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
+      <c r="G2" s="175"/>
+      <c r="H2" s="175"/>
+      <c r="I2" s="175"/>
+      <c r="J2" s="175"/>
+      <c r="K2" s="175"/>
       <c r="L2" s="59" t="s">
         <v>149</v>
       </c>

</xml_diff>

<commit_message>
home from christmas in vegas
</commit_message>
<xml_diff>
--- a/Documents/OMNIXIE_sheets.xlsx
+++ b/Documents/OMNIXIE_sheets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21nic\OneDrive\Desktop\NIXIE\OMNIXIE\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB799917-C225-4D0E-8E1E-FB18979C06B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A935178C-2B01-4956-B09C-D10451DA4829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="227">
   <si>
     <t>A: ADC, A7 (ADC_IN7)</t>
   </si>
@@ -632,12 +632,6 @@
     <t>J6,J7</t>
   </si>
   <si>
-    <t>1x2 2.54mm Pitch Pin Headers</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
     <t xml:space="preserve">CR0603-FX-5101ELF </t>
   </si>
   <si>
@@ -705,6 +699,27 @@
   </si>
   <si>
     <t>Capacitor_SMD:C_0603_1608Metric</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/koa-speer-electronics-inc/RCUCTE/11476561</t>
+  </si>
+  <si>
+    <t>2.54mm Pitch Pin Headers</t>
+  </si>
+  <si>
+    <t>D2, D3</t>
+  </si>
+  <si>
+    <t>Green 525nm LED Indication - Discrete 3.2V 0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>150060GS73220</t>
+  </si>
+  <si>
+    <t>Semiconductors</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -841,7 +856,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -938,8 +953,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="42">
+  <borders count="48">
     <border>
       <left/>
       <right/>
@@ -1175,43 +1202,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1348,19 +1344,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -1464,16 +1447,132 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="double">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1483,7 +1582,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="237">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1582,40 +1681,40 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1628,7 +1727,7 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
@@ -1649,12 +1748,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1685,148 +1778,117 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
@@ -1834,97 +1896,257 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1936,6 +2158,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCCCCFF"/>
       <color rgb="FFCC99FF"/>
     </mruColors>
   </colors>
@@ -2443,7 +2666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10C7034E-99F6-4C64-9A78-788C06E81851}">
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -2467,17 +2690,17 @@
       <c r="B1" s="40">
         <v>1</v>
       </c>
-      <c r="C1" s="169" t="s">
+      <c r="C1" s="149" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="170"/>
-      <c r="E1" s="170"/>
-      <c r="F1" s="170"/>
-      <c r="G1" s="170"/>
-      <c r="H1" s="170"/>
-      <c r="I1" s="170"/>
-      <c r="J1" s="170"/>
-      <c r="K1" s="171"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="151"/>
       <c r="L1" s="36"/>
       <c r="M1" s="36"/>
     </row>
@@ -2488,15 +2711,15 @@
       <c r="B2" s="40">
         <v>1</v>
       </c>
-      <c r="C2" s="172"/>
-      <c r="D2" s="173"/>
-      <c r="E2" s="173"/>
-      <c r="F2" s="173"/>
-      <c r="G2" s="173"/>
-      <c r="H2" s="173"/>
-      <c r="I2" s="173"/>
-      <c r="J2" s="173"/>
-      <c r="K2" s="174"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="153"/>
+      <c r="E2" s="153"/>
+      <c r="F2" s="153"/>
+      <c r="G2" s="153"/>
+      <c r="H2" s="153"/>
+      <c r="I2" s="153"/>
+      <c r="J2" s="153"/>
+      <c r="K2" s="154"/>
       <c r="L2" s="36"/>
       <c r="M2" s="36"/>
     </row>
@@ -2507,182 +2730,182 @@
       <c r="B3" s="40">
         <v>1</v>
       </c>
-      <c r="C3" s="163" t="s">
+      <c r="C3" s="146" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="164"/>
-      <c r="E3" s="164"/>
-      <c r="F3" s="164"/>
-      <c r="G3" s="164"/>
-      <c r="H3" s="164"/>
-      <c r="I3" s="164"/>
-      <c r="J3" s="164"/>
-      <c r="K3" s="165"/>
+      <c r="D3" s="147"/>
+      <c r="E3" s="147"/>
+      <c r="F3" s="147"/>
+      <c r="G3" s="147"/>
+      <c r="H3" s="147"/>
+      <c r="I3" s="147"/>
+      <c r="J3" s="147"/>
+      <c r="K3" s="148"/>
       <c r="L3" s="36"/>
       <c r="M3" s="36"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="147" t="s">
+      <c r="A4" s="132" t="s">
         <v>140</v>
       </c>
-      <c r="B4" s="148">
-        <v>46009</v>
-      </c>
-      <c r="C4" s="166"/>
-      <c r="D4" s="167"/>
-      <c r="E4" s="167"/>
-      <c r="F4" s="167"/>
-      <c r="G4" s="167"/>
-      <c r="H4" s="167"/>
-      <c r="I4" s="167"/>
-      <c r="J4" s="167"/>
-      <c r="K4" s="168"/>
+      <c r="B4" s="133">
+        <v>46017</v>
+      </c>
+      <c r="C4" s="171"/>
+      <c r="D4" s="172"/>
+      <c r="E4" s="172"/>
+      <c r="F4" s="172"/>
+      <c r="G4" s="172"/>
+      <c r="H4" s="172"/>
+      <c r="I4" s="172"/>
+      <c r="J4" s="172"/>
+      <c r="K4" s="173"/>
       <c r="L4" s="36"/>
       <c r="M4" s="36"/>
     </row>
-    <row r="5" spans="1:13" s="122" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="157" t="s">
+    <row r="5" spans="1:13" s="109" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="174" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="158" t="s">
+      <c r="B5" s="175" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="158" t="s">
+      <c r="C5" s="175" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="158" t="s">
+      <c r="D5" s="175" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="158" t="s">
+      <c r="E5" s="175" t="s">
         <v>165</v>
       </c>
-      <c r="F5" s="158" t="s">
+      <c r="F5" s="175" t="s">
         <v>145</v>
       </c>
-      <c r="G5" s="159" t="s">
+      <c r="G5" s="176" t="s">
         <v>95</v>
       </c>
-      <c r="H5" s="158" t="s">
+      <c r="H5" s="175" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="158" t="s">
+      <c r="I5" s="175" t="s">
         <v>136</v>
       </c>
-      <c r="J5" s="158" t="s">
+      <c r="J5" s="175" t="s">
         <v>137</v>
       </c>
-      <c r="K5" s="160" t="s">
+      <c r="K5" s="177" t="s">
         <v>138</v>
       </c>
-      <c r="L5" s="121"/>
-      <c r="M5" s="121"/>
+      <c r="L5" s="108"/>
+      <c r="M5" s="108"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="149" t="s">
+      <c r="A6" s="134" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="150">
+      <c r="B6" s="135">
         <v>1</v>
       </c>
-      <c r="C6" s="150" t="s">
+      <c r="C6" s="135" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="151" t="s">
+      <c r="D6" s="136" t="s">
         <v>186</v>
       </c>
-      <c r="E6" s="152" t="s">
+      <c r="E6" s="137" t="s">
         <v>166</v>
       </c>
-      <c r="F6" s="153"/>
-      <c r="G6" s="154" t="s">
+      <c r="F6" s="138"/>
+      <c r="G6" s="139" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="155"/>
-      <c r="I6" s="155"/>
-      <c r="J6" s="155"/>
-      <c r="K6" s="156"/>
+      <c r="H6" s="140"/>
+      <c r="I6" s="140"/>
+      <c r="J6" s="140"/>
+      <c r="K6" s="141"/>
       <c r="L6" s="36"/>
       <c r="M6" s="36"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="97"/>
-      <c r="B7" s="98">
+      <c r="A7" s="84"/>
+      <c r="B7" s="85">
         <v>1</v>
       </c>
-      <c r="C7" s="98" t="s">
+      <c r="C7" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="99" t="s">
+      <c r="D7" s="86" t="s">
         <v>187</v>
       </c>
-      <c r="E7" s="100" t="s">
+      <c r="E7" s="87" t="s">
         <v>166</v>
       </c>
-      <c r="F7" s="101"/>
-      <c r="G7" s="102" t="s">
+      <c r="F7" s="88"/>
+      <c r="G7" s="89" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="103"/>
-      <c r="I7" s="103"/>
-      <c r="J7" s="103"/>
-      <c r="K7" s="104"/>
+      <c r="H7" s="90"/>
+      <c r="I7" s="90"/>
+      <c r="J7" s="90"/>
+      <c r="K7" s="91"/>
       <c r="L7" s="36"/>
       <c r="M7" s="36"/>
     </row>
-    <row r="8" spans="1:13" s="122" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="113"/>
-      <c r="B8" s="114">
+    <row r="8" spans="1:13" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="100"/>
+      <c r="B8" s="101">
         <v>1</v>
       </c>
-      <c r="C8" s="114" t="s">
+      <c r="C8" s="101" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="115" t="s">
+      <c r="D8" s="102" t="s">
         <v>188</v>
       </c>
-      <c r="E8" s="116" t="s">
+      <c r="E8" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="F8" s="117"/>
-      <c r="G8" s="118" t="s">
+      <c r="F8" s="104"/>
+      <c r="G8" s="105" t="s">
         <v>104</v>
       </c>
-      <c r="H8" s="119"/>
-      <c r="I8" s="119"/>
-      <c r="J8" s="119"/>
-      <c r="K8" s="120"/>
-      <c r="L8" s="121"/>
-      <c r="M8" s="121"/>
+      <c r="H8" s="106"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="106"/>
+      <c r="K8" s="107"/>
+      <c r="L8" s="108"/>
+      <c r="M8" s="108"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="105" t="s">
+      <c r="A9" s="92" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="106">
+      <c r="B9" s="93">
         <v>1</v>
       </c>
-      <c r="C9" s="162" t="s">
-        <v>208</v>
-      </c>
-      <c r="D9" s="107" t="s">
+      <c r="C9" s="143" t="s">
+        <v>206</v>
+      </c>
+      <c r="D9" s="94" t="s">
         <v>189</v>
       </c>
-      <c r="E9" s="108" t="s">
+      <c r="E9" s="95" t="s">
         <v>166</v>
       </c>
-      <c r="F9" s="109"/>
-      <c r="G9" s="110" t="s">
+      <c r="F9" s="96"/>
+      <c r="G9" s="97" t="s">
         <v>103</v>
       </c>
-      <c r="H9" s="111"/>
-      <c r="I9" s="111"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="112"/>
+      <c r="H9" s="98"/>
+      <c r="I9" s="98"/>
+      <c r="J9" s="98"/>
+      <c r="K9" s="99"/>
       <c r="L9" s="36"/>
       <c r="M9" s="36"/>
     </row>
     <row r="10" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="84"/>
+      <c r="A10" s="79"/>
       <c r="B10" s="62">
         <v>2</v>
       </c>
@@ -2695,21 +2918,19 @@
       <c r="E10" s="64" t="s">
         <v>166</v>
       </c>
-      <c r="F10" s="65" t="s">
-        <v>198</v>
-      </c>
+      <c r="F10" s="65"/>
       <c r="G10" s="66" t="s">
-        <v>197</v>
+        <v>221</v>
       </c>
       <c r="H10" s="67"/>
       <c r="I10" s="67"/>
       <c r="J10" s="67"/>
-      <c r="K10" s="85"/>
+      <c r="K10" s="80"/>
       <c r="L10" s="61"/>
       <c r="M10" s="61"/>
     </row>
     <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="86"/>
+      <c r="A11" s="81"/>
       <c r="B11" s="62">
         <v>1</v>
       </c>
@@ -2729,527 +2950,526 @@
       <c r="H11" s="67"/>
       <c r="I11" s="67"/>
       <c r="J11" s="67"/>
-      <c r="K11" s="85"/>
+      <c r="K11" s="80"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="86"/>
-      <c r="B12" s="62">
+      <c r="A12" s="110"/>
+      <c r="B12" s="111">
         <v>2</v>
       </c>
-      <c r="C12" s="62" t="s">
+      <c r="C12" s="111" t="s">
         <v>101</v>
       </c>
-      <c r="D12" s="68" t="s">
+      <c r="D12" s="188" t="s">
         <v>190</v>
       </c>
-      <c r="E12" s="64" t="s">
+      <c r="E12" s="112" t="s">
         <v>166</v>
       </c>
-      <c r="F12" s="65"/>
-      <c r="G12" s="66" t="s">
+      <c r="F12" s="113"/>
+      <c r="G12" s="114" t="s">
         <v>102</v>
       </c>
-      <c r="H12" s="67"/>
-      <c r="I12" s="67"/>
-      <c r="J12" s="67"/>
-      <c r="K12" s="85"/>
+      <c r="H12" s="115"/>
+      <c r="I12" s="115"/>
+      <c r="J12" s="115"/>
+      <c r="K12" s="116"/>
       <c r="L12" s="36"/>
       <c r="M12" s="36"/>
     </row>
-    <row r="13" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="86"/>
-      <c r="B13" s="62">
+    <row r="13" spans="1:13" s="198" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="125"/>
+      <c r="B13" s="126">
         <v>1</v>
       </c>
-      <c r="C13" s="62" t="s">
+      <c r="C13" s="126" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="68" t="s">
-        <v>211</v>
-      </c>
-      <c r="E13" s="64" t="s">
+      <c r="D13" s="196" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" s="127" t="s">
         <v>166</v>
       </c>
-      <c r="F13" s="65"/>
-      <c r="G13" s="66" t="s">
-        <v>209</v>
-      </c>
-      <c r="H13" s="67"/>
-      <c r="I13" s="67"/>
-      <c r="J13" s="67"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="61"/>
-      <c r="M13" s="61"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="86"/>
-      <c r="B14" s="62">
+      <c r="F13" s="128"/>
+      <c r="G13" s="129" t="s">
+        <v>207</v>
+      </c>
+      <c r="H13" s="130"/>
+      <c r="I13" s="130"/>
+      <c r="J13" s="130"/>
+      <c r="K13" s="131"/>
+      <c r="L13" s="197"/>
+      <c r="M13" s="197"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="164" t="s">
+        <v>225</v>
+      </c>
+      <c r="B14" s="189">
         <v>1</v>
       </c>
-      <c r="C14" s="62" t="s">
+      <c r="C14" s="189" t="s">
         <v>110</v>
       </c>
-      <c r="D14" s="69" t="s">
+      <c r="D14" s="190" t="s">
         <v>193</v>
       </c>
-      <c r="E14" s="64" t="s">
+      <c r="E14" s="191" t="s">
         <v>166</v>
       </c>
-      <c r="F14" s="65"/>
-      <c r="G14" s="66" t="s">
+      <c r="F14" s="192"/>
+      <c r="G14" s="193" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="67"/>
-      <c r="I14" s="67"/>
-      <c r="J14" s="67"/>
-      <c r="K14" s="85"/>
+      <c r="H14" s="194"/>
+      <c r="I14" s="194"/>
+      <c r="J14" s="194"/>
+      <c r="K14" s="195"/>
       <c r="L14" s="36"/>
       <c r="M14" s="36"/>
     </row>
     <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="86"/>
-      <c r="B15" s="62">
+      <c r="A15" s="156"/>
+      <c r="B15" s="157">
         <v>12</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="157" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="69" t="s">
+      <c r="D15" s="158" t="s">
         <v>192</v>
       </c>
-      <c r="E15" s="64" t="s">
+      <c r="E15" s="159" t="s">
         <v>166</v>
       </c>
-      <c r="F15" s="65"/>
-      <c r="G15" s="66" t="s">
+      <c r="F15" s="160"/>
+      <c r="G15" s="161" t="s">
         <v>134</v>
       </c>
-      <c r="H15" s="67"/>
-      <c r="I15" s="67"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="85"/>
+      <c r="H15" s="162"/>
+      <c r="I15" s="162"/>
+      <c r="J15" s="162"/>
+      <c r="K15" s="163"/>
       <c r="L15" s="36"/>
       <c r="M15" s="36"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="123"/>
-      <c r="B16" s="124">
+    <row r="16" spans="1:13" s="210" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="156"/>
+      <c r="B16" s="157">
         <v>1</v>
       </c>
-      <c r="C16" s="124" t="s">
-        <v>113</v>
-      </c>
-      <c r="D16" s="125" t="s">
-        <v>194</v>
-      </c>
-      <c r="E16" s="126" t="s">
+      <c r="C16" s="157" t="s">
+        <v>121</v>
+      </c>
+      <c r="D16" s="158" t="s">
+        <v>195</v>
+      </c>
+      <c r="E16" s="159" t="s">
         <v>166</v>
       </c>
-      <c r="F16" s="127"/>
-      <c r="G16" s="128" t="s">
-        <v>123</v>
-      </c>
-      <c r="H16" s="129"/>
-      <c r="I16" s="129"/>
-      <c r="J16" s="129"/>
-      <c r="K16" s="130"/>
-      <c r="L16" s="36"/>
-      <c r="M16" s="36"/>
-    </row>
-    <row r="17" spans="1:13" s="122" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="139"/>
-      <c r="B17" s="140">
+      <c r="F16" s="160"/>
+      <c r="G16" s="161" t="s">
+        <v>130</v>
+      </c>
+      <c r="H16" s="162"/>
+      <c r="I16" s="162"/>
+      <c r="J16" s="162"/>
+      <c r="K16" s="163"/>
+      <c r="L16" s="209"/>
+      <c r="M16" s="209"/>
+    </row>
+    <row r="17" spans="1:13" s="208" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="199"/>
+      <c r="B17" s="200">
+        <v>2</v>
+      </c>
+      <c r="C17" s="200" t="s">
+        <v>224</v>
+      </c>
+      <c r="D17" s="201" t="s">
+        <v>222</v>
+      </c>
+      <c r="E17" s="202" t="s">
+        <v>166</v>
+      </c>
+      <c r="F17" s="203"/>
+      <c r="G17" s="204" t="s">
+        <v>223</v>
+      </c>
+      <c r="H17" s="205"/>
+      <c r="I17" s="205"/>
+      <c r="J17" s="205"/>
+      <c r="K17" s="206"/>
+      <c r="L17" s="207"/>
+      <c r="M17" s="207"/>
+    </row>
+    <row r="18" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="117" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="118">
         <v>1</v>
       </c>
-      <c r="C17" s="140" t="s">
-        <v>121</v>
-      </c>
-      <c r="D17" s="141" t="s">
-        <v>195</v>
-      </c>
-      <c r="E17" s="142" t="s">
-        <v>166</v>
-      </c>
-      <c r="F17" s="143"/>
-      <c r="G17" s="144" t="s">
-        <v>130</v>
-      </c>
-      <c r="H17" s="145"/>
-      <c r="I17" s="145"/>
-      <c r="J17" s="145"/>
-      <c r="K17" s="146"/>
-      <c r="L17" s="121"/>
-      <c r="M17" s="121"/>
-    </row>
-    <row r="18" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="131" t="s">
-        <v>185</v>
-      </c>
-      <c r="B18" s="132">
-        <v>1</v>
-      </c>
-      <c r="C18" s="132" t="s">
+      <c r="C18" s="118" t="s">
         <v>158</v>
       </c>
-      <c r="D18" s="133" t="s">
+      <c r="D18" s="119" t="s">
         <v>160</v>
       </c>
-      <c r="E18" s="134" t="s">
+      <c r="E18" s="120" t="s">
         <v>167</v>
       </c>
-      <c r="F18" s="135"/>
-      <c r="G18" s="136" t="s">
+      <c r="F18" s="121"/>
+      <c r="G18" s="122" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="176" t="s">
+      <c r="H18" s="144" t="s">
         <v>183</v>
       </c>
-      <c r="I18" s="137"/>
-      <c r="J18" s="137"/>
-      <c r="K18" s="138"/>
+      <c r="I18" s="123"/>
+      <c r="J18" s="123"/>
+      <c r="K18" s="124"/>
       <c r="L18" s="36"/>
       <c r="M18" s="36"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="87"/>
-      <c r="B19" s="71">
+      <c r="A19" s="82"/>
+      <c r="B19" s="69">
         <v>1</v>
       </c>
-      <c r="C19" s="71" t="s">
-        <v>206</v>
-      </c>
-      <c r="D19" s="73" t="s">
+      <c r="C19" s="69" t="s">
+        <v>204</v>
+      </c>
+      <c r="D19" s="71" t="s">
         <v>161</v>
       </c>
-      <c r="E19" s="74" t="s">
+      <c r="E19" s="72" t="s">
         <v>168</v>
       </c>
-      <c r="F19" s="75"/>
-      <c r="G19" s="72" t="s">
-        <v>207</v>
-      </c>
-      <c r="H19" s="177" t="s">
+      <c r="F19" s="73"/>
+      <c r="G19" s="70" t="s">
+        <v>205</v>
+      </c>
+      <c r="H19" s="145" t="s">
         <v>184</v>
       </c>
-      <c r="I19" s="70"/>
-      <c r="J19" s="70"/>
-      <c r="K19" s="88"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="68"/>
+      <c r="K19" s="83"/>
       <c r="L19" s="36"/>
       <c r="M19" s="36"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="87"/>
-      <c r="B20" s="71">
+      <c r="A20" s="82"/>
+      <c r="B20" s="69">
         <v>1</v>
       </c>
-      <c r="C20" s="71" t="s">
-        <v>212</v>
-      </c>
-      <c r="D20" s="73" t="s">
+      <c r="C20" s="69" t="s">
+        <v>210</v>
+      </c>
+      <c r="D20" s="71" t="s">
         <v>162</v>
       </c>
-      <c r="E20" s="74" t="s">
+      <c r="E20" s="72" t="s">
         <v>169</v>
       </c>
-      <c r="F20" s="75"/>
-      <c r="G20" s="76" t="s">
-        <v>213</v>
-      </c>
-      <c r="H20" s="177" t="s">
-        <v>221</v>
-      </c>
-      <c r="I20" s="70"/>
-      <c r="J20" s="70"/>
-      <c r="K20" s="88"/>
+      <c r="F20" s="73"/>
+      <c r="G20" s="74" t="s">
+        <v>211</v>
+      </c>
+      <c r="H20" s="145" t="s">
+        <v>219</v>
+      </c>
+      <c r="I20" s="68"/>
+      <c r="J20" s="68"/>
+      <c r="K20" s="83"/>
       <c r="L20" s="36"/>
       <c r="M20" s="36"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="87"/>
-      <c r="B21" s="77">
+      <c r="A21" s="82"/>
+      <c r="B21" s="75">
         <v>2</v>
       </c>
-      <c r="C21" s="77" t="s">
+      <c r="C21" s="75" t="s">
+        <v>216</v>
+      </c>
+      <c r="D21" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="E21" s="72" t="s">
         <v>218</v>
       </c>
-      <c r="D21" s="78" t="s">
-        <v>170</v>
-      </c>
-      <c r="E21" s="74" t="s">
-        <v>220</v>
-      </c>
-      <c r="F21" s="79"/>
-      <c r="G21" s="80" t="s">
-        <v>219</v>
-      </c>
-      <c r="H21" s="177" t="s">
+      <c r="F21" s="77"/>
+      <c r="G21" s="78" t="s">
+        <v>217</v>
+      </c>
+      <c r="H21" s="145" t="s">
         <v>182</v>
       </c>
-      <c r="I21" s="70"/>
-      <c r="J21" s="70"/>
-      <c r="K21" s="88"/>
+      <c r="I21" s="68"/>
+      <c r="J21" s="68"/>
+      <c r="K21" s="83"/>
       <c r="L21" s="36"/>
       <c r="M21" s="36"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="87"/>
-      <c r="B22" s="77">
+      <c r="A22" s="82"/>
+      <c r="B22" s="75">
         <v>1</v>
       </c>
-      <c r="C22" s="71" t="s">
-        <v>204</v>
-      </c>
-      <c r="D22" s="78" t="s">
+      <c r="C22" s="69" t="s">
+        <v>202</v>
+      </c>
+      <c r="D22" s="76" t="s">
         <v>163</v>
       </c>
-      <c r="E22" s="74" t="s">
+      <c r="E22" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="F22" s="75"/>
-      <c r="G22" s="76" t="s">
-        <v>203</v>
-      </c>
-      <c r="H22" s="177" t="s">
+      <c r="F22" s="73"/>
+      <c r="G22" s="74" t="s">
+        <v>201</v>
+      </c>
+      <c r="H22" s="145" t="s">
         <v>181</v>
       </c>
-      <c r="I22" s="70"/>
-      <c r="J22" s="70"/>
-      <c r="K22" s="88"/>
+      <c r="I22" s="68"/>
+      <c r="J22" s="68"/>
+      <c r="K22" s="83"/>
       <c r="L22" s="36"/>
       <c r="M22" s="36"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="87"/>
-      <c r="B23" s="77">
+      <c r="A23" s="82"/>
+      <c r="B23" s="75">
         <v>1</v>
       </c>
-      <c r="C23" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="D23" s="78" t="s">
+      <c r="C23" s="69" t="s">
+        <v>214</v>
+      </c>
+      <c r="D23" s="76" t="s">
         <v>164</v>
       </c>
-      <c r="E23" s="74" t="s">
+      <c r="E23" s="72" t="s">
         <v>172</v>
       </c>
-      <c r="F23" s="75"/>
-      <c r="G23" s="76" t="s">
-        <v>217</v>
-      </c>
-      <c r="H23" s="177" t="s">
+      <c r="F23" s="73"/>
+      <c r="G23" s="74" t="s">
+        <v>215</v>
+      </c>
+      <c r="H23" s="145" t="s">
         <v>180</v>
       </c>
-      <c r="I23" s="70"/>
-      <c r="J23" s="70"/>
-      <c r="K23" s="88"/>
+      <c r="I23" s="68"/>
+      <c r="J23" s="68"/>
+      <c r="K23" s="83"/>
       <c r="L23" s="36"/>
       <c r="M23" s="36"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="87"/>
-      <c r="B24" s="77">
+      <c r="A24" s="82"/>
+      <c r="B24" s="75">
         <v>2</v>
       </c>
-      <c r="C24" s="161">
+      <c r="C24" s="142">
         <v>560112110017</v>
       </c>
-      <c r="D24" s="78" t="s">
+      <c r="D24" s="76" t="s">
         <v>173</v>
       </c>
-      <c r="E24" s="74">
+      <c r="E24" s="72">
         <v>47</v>
       </c>
-      <c r="F24" s="79"/>
-      <c r="G24" s="80" t="s">
-        <v>205</v>
-      </c>
-      <c r="H24" s="177" t="s">
+      <c r="F24" s="77"/>
+      <c r="G24" s="78" t="s">
+        <v>203</v>
+      </c>
+      <c r="H24" s="145" t="s">
         <v>180</v>
       </c>
-      <c r="I24" s="70"/>
-      <c r="J24" s="70"/>
-      <c r="K24" s="88"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
+      <c r="K24" s="83"/>
       <c r="L24" s="36"/>
       <c r="M24" s="36"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="87"/>
-      <c r="B25" s="77">
+      <c r="A25" s="82"/>
+      <c r="B25" s="75">
         <v>2</v>
       </c>
-      <c r="C25" s="77" t="s">
-        <v>214</v>
-      </c>
-      <c r="D25" s="78" t="s">
+      <c r="C25" s="75" t="s">
+        <v>212</v>
+      </c>
+      <c r="D25" s="76" t="s">
         <v>174</v>
       </c>
-      <c r="E25" s="74" t="s">
+      <c r="E25" s="72" t="s">
         <v>175</v>
       </c>
-      <c r="F25" s="79"/>
-      <c r="G25" s="80" t="s">
-        <v>215</v>
-      </c>
-      <c r="H25" s="177" t="s">
+      <c r="F25" s="77"/>
+      <c r="G25" s="78" t="s">
+        <v>213</v>
+      </c>
+      <c r="H25" s="145" t="s">
         <v>182</v>
       </c>
-      <c r="I25" s="70"/>
-      <c r="J25" s="70"/>
-      <c r="K25" s="88"/>
+      <c r="I25" s="68"/>
+      <c r="J25" s="68"/>
+      <c r="K25" s="83"/>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="87"/>
-      <c r="B26" s="77">
+      <c r="A26" s="211"/>
+      <c r="B26" s="212">
         <v>2</v>
       </c>
-      <c r="C26" s="77" t="s">
-        <v>199</v>
-      </c>
-      <c r="D26" s="78" t="s">
+      <c r="C26" s="212" t="s">
+        <v>197</v>
+      </c>
+      <c r="D26" s="213" t="s">
         <v>176</v>
       </c>
-      <c r="E26" s="74" t="s">
+      <c r="E26" s="214" t="s">
         <v>177</v>
       </c>
-      <c r="F26" s="79"/>
-      <c r="G26" s="81" t="s">
-        <v>200</v>
-      </c>
-      <c r="H26" s="177" t="s">
+      <c r="F26" s="215"/>
+      <c r="G26" s="216" t="s">
+        <v>198</v>
+      </c>
+      <c r="H26" s="217" t="s">
         <v>182</v>
       </c>
-      <c r="I26" s="70"/>
-      <c r="J26" s="70"/>
-      <c r="K26" s="88"/>
+      <c r="I26" s="218"/>
+      <c r="J26" s="218"/>
+      <c r="K26" s="219"/>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="87"/>
-      <c r="B27" s="77">
+    <row r="27" spans="1:13" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="228"/>
+      <c r="B27" s="229">
         <v>1</v>
       </c>
-      <c r="C27" s="77" t="s">
-        <v>201</v>
-      </c>
-      <c r="D27" s="78" t="s">
+      <c r="C27" s="229" t="s">
+        <v>199</v>
+      </c>
+      <c r="D27" s="230" t="s">
         <v>178</v>
       </c>
-      <c r="E27" s="74" t="s">
+      <c r="E27" s="231" t="s">
         <v>179</v>
       </c>
-      <c r="F27" s="79"/>
-      <c r="G27" s="81" t="s">
-        <v>202</v>
-      </c>
-      <c r="H27" s="177" t="s">
+      <c r="F27" s="232"/>
+      <c r="G27" s="233" t="s">
+        <v>200</v>
+      </c>
+      <c r="H27" s="234" t="s">
         <v>180</v>
       </c>
-      <c r="I27" s="70"/>
-      <c r="J27" s="70"/>
-      <c r="K27" s="88"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="87"/>
-      <c r="B28" s="82"/>
-      <c r="C28" s="72"/>
-      <c r="D28" s="83"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="72"/>
-      <c r="H28" s="70"/>
-      <c r="I28" s="70"/>
-      <c r="J28" s="70"/>
-      <c r="K28" s="88"/>
+      <c r="I27" s="235"/>
+      <c r="J27" s="235"/>
+      <c r="K27" s="236"/>
+      <c r="L27" s="108"/>
+      <c r="M27" s="108"/>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="220" t="s">
+        <v>226</v>
+      </c>
+      <c r="B28" s="221">
+        <v>1</v>
+      </c>
+      <c r="C28" s="221" t="s">
+        <v>113</v>
+      </c>
+      <c r="D28" s="222" t="s">
+        <v>194</v>
+      </c>
+      <c r="E28" s="223" t="s">
+        <v>166</v>
+      </c>
+      <c r="F28" s="224"/>
+      <c r="G28" s="225" t="s">
+        <v>123</v>
+      </c>
+      <c r="H28" s="226"/>
+      <c r="I28" s="226"/>
+      <c r="J28" s="226"/>
+      <c r="K28" s="227"/>
       <c r="L28" s="36"/>
       <c r="M28" s="36"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="87"/>
-      <c r="B29" s="82"/>
-      <c r="C29" s="70"/>
-      <c r="D29" s="83"/>
-      <c r="E29" s="70"/>
-      <c r="F29" s="75"/>
-      <c r="G29" s="72"/>
-      <c r="H29" s="70"/>
-      <c r="I29" s="70"/>
-      <c r="J29" s="70"/>
-      <c r="K29" s="88"/>
+      <c r="A29" s="178"/>
+      <c r="B29" s="166"/>
+      <c r="C29" s="167"/>
+      <c r="D29" s="168"/>
+      <c r="E29" s="165"/>
+      <c r="F29" s="169"/>
+      <c r="G29" s="170"/>
+      <c r="H29" s="165"/>
+      <c r="I29" s="165"/>
+      <c r="J29" s="165"/>
+      <c r="K29" s="179"/>
       <c r="L29" s="36"/>
       <c r="M29" s="36"/>
     </row>
-    <row r="30" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="89"/>
-      <c r="B30" s="90"/>
-      <c r="C30" s="91"/>
-      <c r="D30" s="92"/>
-      <c r="E30" s="93"/>
-      <c r="F30" s="94"/>
-      <c r="G30" s="95"/>
-      <c r="H30" s="93"/>
-      <c r="I30" s="93"/>
-      <c r="J30" s="93"/>
-      <c r="K30" s="96"/>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="178"/>
+      <c r="B30" s="165"/>
+      <c r="C30" s="165"/>
+      <c r="D30" s="165"/>
+      <c r="E30" s="165"/>
+      <c r="F30" s="165"/>
+      <c r="G30" s="165"/>
+      <c r="H30" s="165"/>
+      <c r="I30" s="165"/>
+      <c r="J30" s="165"/>
+      <c r="K30" s="179"/>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="33"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="36"/>
+      <c r="A31" s="178"/>
+      <c r="B31" s="165"/>
+      <c r="C31" s="165"/>
+      <c r="D31" s="165"/>
+      <c r="E31" s="165"/>
+      <c r="F31" s="165"/>
+      <c r="G31" s="165"/>
+      <c r="H31" s="165"/>
+      <c r="I31" s="165"/>
+      <c r="J31" s="165"/>
+      <c r="K31" s="179"/>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" s="33"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="33"/>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="33"/>
-      <c r="J32" s="33"/>
-      <c r="K32" s="36"/>
-      <c r="L32" s="36"/>
-      <c r="M32" s="36"/>
-    </row>
-    <row r="33" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="86"/>
-      <c r="B33" s="62">
+    <row r="32" spans="1:13" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="180"/>
+      <c r="B32" s="181">
         <v>1</v>
       </c>
-      <c r="C33" s="62" t="s">
+      <c r="C32" s="181" t="s">
         <v>119</v>
       </c>
-      <c r="D33" s="68"/>
-      <c r="E33" s="64" t="s">
+      <c r="D32" s="182"/>
+      <c r="E32" s="183" t="s">
         <v>166</v>
       </c>
-      <c r="F33" s="65"/>
-      <c r="G33" s="66" t="s">
-        <v>210</v>
-      </c>
-      <c r="H33" s="67"/>
-      <c r="I33" s="67"/>
-      <c r="J33" s="67"/>
-      <c r="K33" s="85"/>
-      <c r="L33" s="61"/>
-      <c r="M33" s="61"/>
+      <c r="F32" s="184"/>
+      <c r="G32" s="185" t="s">
+        <v>208</v>
+      </c>
+      <c r="H32" s="186"/>
+      <c r="I32" s="186"/>
+      <c r="J32" s="186"/>
+      <c r="K32" s="187"/>
+      <c r="L32" s="61"/>
+      <c r="M32" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3283,14 +3503,14 @@
       <c r="E2" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="175" t="s">
+      <c r="F2" s="155" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="175"/>
-      <c r="H2" s="175"/>
-      <c r="I2" s="175"/>
-      <c r="J2" s="175"/>
-      <c r="K2" s="175"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="155"/>
+      <c r="K2" s="155"/>
       <c r="L2" s="59" t="s">
         <v>149</v>
       </c>
@@ -3803,7 +4023,7 @@
       <c r="L22" s="56"/>
     </row>
     <row r="25" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="E25" t="s">
+      <c r="E25" s="57" t="s">
         <v>153</v>
       </c>
     </row>
@@ -3833,10 +4053,11 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E27" r:id="rId1" xr:uid="{E0F6383B-4BDA-4ACA-9049-DCAA748F9F7E}"/>
+    <hyperlink ref="E25" r:id="rId2" xr:uid="{EB1DDABE-E978-4224-A476-73147F7CBB33}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
-  <drawing r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
 
@@ -3948,7 +4169,8 @@
   <dimension ref="B3:H26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
@@ -4001,6 +4223,11 @@
       <c r="F8" s="33"/>
       <c r="G8" s="35" t="s">
         <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="19" spans="4:8" ht="23.25" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
separated proto from production version with actual footprints
</commit_message>
<xml_diff>
--- a/Documents/OMNIXIE_sheets.xlsx
+++ b/Documents/OMNIXIE_sheets.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21nic\OneDrive\Desktop\NIXIE\OMNIXIE\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A935178C-2B01-4956-B09C-D10451DA4829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E1B675-60BB-46F2-B3B3-C2EC7950E151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="BOM" sheetId="4" r:id="rId1"/>
-    <sheet name="CH32V003F4U6 PIN FUNCTIONS" sheetId="1" r:id="rId2"/>
-    <sheet name="COST ESTIMATES" sheetId="3" r:id="rId3"/>
-    <sheet name="ARCHIVE" sheetId="5" r:id="rId4"/>
+    <sheet name="PROTOTYPE BOM v1" sheetId="6" r:id="rId1"/>
+    <sheet name="PRODUCTION BOM" sheetId="4" r:id="rId2"/>
+    <sheet name="CH32V003F4U6 PIN FUNCTIONS" sheetId="1" r:id="rId3"/>
+    <sheet name="COST ESTIMATES" sheetId="3" r:id="rId4"/>
+    <sheet name="ARCHIVE" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="240">
   <si>
     <t>A: ADC, A7 (ADC_IN7)</t>
   </si>
@@ -720,6 +721,45 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>IN12-A sockets purchased</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B09D2VQR3Q</t>
+  </si>
+  <si>
+    <t>Package_DFN_QFN:QFN-20-1EP_3x3mm_P0.4mm_EP1.65x1.65mm</t>
+  </si>
+  <si>
+    <t>Package_DFN_QFN:TQFN-24-1EP_4x4mm_P0.5mm_EP2.1x2.1mm_ThermalVias</t>
+  </si>
+  <si>
+    <t>Package_TO_SOT_SMD:SOT-23-3</t>
+  </si>
+  <si>
+    <t>TestPoint:TestPoint_Keystone_5005-5009_Compact</t>
+  </si>
+  <si>
+    <t>TO BUY</t>
+  </si>
+  <si>
+    <t>PROCURED</t>
+  </si>
+  <si>
+    <t>_0805</t>
+  </si>
+  <si>
+    <t>Package_TO_SOT_SMD:SOT-223-3_TabPin2</t>
+  </si>
+  <si>
+    <t>OMNIXIE:SK3200AFL</t>
+  </si>
+  <si>
+    <t>LED_SMD:LED_0603_1608Metric</t>
+  </si>
+  <si>
+    <t>J1,J6</t>
   </si>
 </sst>
 </file>
@@ -729,7 +769,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -855,8 +895,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -965,6 +1011,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="48">
     <border>
@@ -1582,7 +1634,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="237">
+  <cellXfs count="281">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1840,7 +1892,6 @@
     <xf numFmtId="0" fontId="8" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1926,45 +1977,6 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1985,9 +1997,6 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1998,18 +2007,6 @@
     <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2022,7 +2019,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2147,6 +2143,229 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2154,10 +2373,36 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="3" xr:uid="{B93126DE-0D01-4C50-8056-E448E7756006}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF00FF00"/>
       <color rgb="FFCCCCFF"/>
       <color rgb="FFCC99FF"/>
     </mruColors>
@@ -2401,6 +2646,23 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2665,6 +2927,1004 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE706952-430C-44AA-84E6-C88695E38A9F}">
+  <dimension ref="A1:O31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="121.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="39"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="40">
+        <v>1</v>
+      </c>
+      <c r="E1" s="228" t="s">
+        <v>139</v>
+      </c>
+      <c r="F1" s="229"/>
+      <c r="G1" s="229"/>
+      <c r="H1" s="229"/>
+      <c r="I1" s="229"/>
+      <c r="J1" s="229"/>
+      <c r="K1" s="229"/>
+      <c r="L1" s="229"/>
+      <c r="M1" s="230"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+    </row>
+    <row r="2" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="40">
+        <v>1</v>
+      </c>
+      <c r="E2" s="231"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="232"/>
+      <c r="H2" s="232"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="M2" s="233"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+    </row>
+    <row r="3" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="41"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="40">
+        <v>1</v>
+      </c>
+      <c r="E3" s="222" t="s">
+        <v>141</v>
+      </c>
+      <c r="F3" s="223"/>
+      <c r="G3" s="223"/>
+      <c r="H3" s="223"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
+      <c r="M3" s="224"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="36"/>
+    </row>
+    <row r="4" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="131"/>
+      <c r="B4" s="131"/>
+      <c r="C4" s="131" t="s">
+        <v>140</v>
+      </c>
+      <c r="D4" s="132">
+        <v>46017</v>
+      </c>
+      <c r="E4" s="225"/>
+      <c r="F4" s="226"/>
+      <c r="G4" s="226"/>
+      <c r="H4" s="226"/>
+      <c r="I4" s="226"/>
+      <c r="J4" s="226"/>
+      <c r="K4" s="226"/>
+      <c r="L4" s="226"/>
+      <c r="M4" s="227"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+    </row>
+    <row r="5" spans="1:15" s="109" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="159" t="s">
+        <v>234</v>
+      </c>
+      <c r="B5" s="159" t="s">
+        <v>233</v>
+      </c>
+      <c r="C5" s="159" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="160" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="160" t="s">
+        <v>93</v>
+      </c>
+      <c r="F5" s="160" t="s">
+        <v>107</v>
+      </c>
+      <c r="G5" s="160" t="s">
+        <v>165</v>
+      </c>
+      <c r="H5" s="160" t="s">
+        <v>145</v>
+      </c>
+      <c r="I5" s="161" t="s">
+        <v>95</v>
+      </c>
+      <c r="J5" s="160" t="s">
+        <v>135</v>
+      </c>
+      <c r="K5" s="160" t="s">
+        <v>136</v>
+      </c>
+      <c r="L5" s="160" t="s">
+        <v>137</v>
+      </c>
+      <c r="M5" s="162" t="s">
+        <v>138</v>
+      </c>
+      <c r="N5" s="108"/>
+      <c r="O5" s="108"/>
+    </row>
+    <row r="6" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B6" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="133" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="134">
+        <v>1</v>
+      </c>
+      <c r="E6" s="134" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="135" t="s">
+        <v>186</v>
+      </c>
+      <c r="G6" s="136" t="s">
+        <v>166</v>
+      </c>
+      <c r="H6" s="137"/>
+      <c r="I6" s="138" t="s">
+        <v>105</v>
+      </c>
+      <c r="J6" s="139" t="s">
+        <v>229</v>
+      </c>
+      <c r="K6" s="139"/>
+      <c r="L6" s="139"/>
+      <c r="M6" s="140"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="36"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B7" s="238" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="84"/>
+      <c r="D7" s="85">
+        <v>1</v>
+      </c>
+      <c r="E7" s="85" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="86" t="s">
+        <v>187</v>
+      </c>
+      <c r="G7" s="87" t="s">
+        <v>166</v>
+      </c>
+      <c r="H7" s="88"/>
+      <c r="I7" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="J7" s="90" t="s">
+        <v>230</v>
+      </c>
+      <c r="K7" s="90"/>
+      <c r="L7" s="90"/>
+      <c r="M7" s="91"/>
+      <c r="N7" s="36"/>
+      <c r="O7" s="36"/>
+    </row>
+    <row r="8" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B8" s="239" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="100"/>
+      <c r="D8" s="101">
+        <v>1</v>
+      </c>
+      <c r="E8" s="101" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="102" t="s">
+        <v>188</v>
+      </c>
+      <c r="G8" s="103" t="s">
+        <v>166</v>
+      </c>
+      <c r="H8" s="104"/>
+      <c r="I8" s="105" t="s">
+        <v>104</v>
+      </c>
+      <c r="J8" s="106" t="s">
+        <v>231</v>
+      </c>
+      <c r="K8" s="106"/>
+      <c r="L8" s="106"/>
+      <c r="M8" s="107"/>
+      <c r="N8" s="108"/>
+      <c r="O8" s="108"/>
+    </row>
+    <row r="9" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B9" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="92" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" s="93">
+        <v>1</v>
+      </c>
+      <c r="E9" s="142" t="s">
+        <v>206</v>
+      </c>
+      <c r="F9" s="94" t="s">
+        <v>189</v>
+      </c>
+      <c r="G9" s="95" t="s">
+        <v>166</v>
+      </c>
+      <c r="H9" s="96"/>
+      <c r="I9" s="97" t="s">
+        <v>103</v>
+      </c>
+      <c r="J9" s="98"/>
+      <c r="K9" s="98"/>
+      <c r="L9" s="98"/>
+      <c r="M9" s="99"/>
+      <c r="N9" s="36"/>
+      <c r="O9" s="36"/>
+    </row>
+    <row r="10" spans="1:15" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="240" t="b">
+        <v>0</v>
+      </c>
+      <c r="C10" s="79"/>
+      <c r="D10" s="62">
+        <v>2</v>
+      </c>
+      <c r="E10" s="62" t="s">
+        <v>166</v>
+      </c>
+      <c r="F10" s="63" t="s">
+        <v>239</v>
+      </c>
+      <c r="G10" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="H10" s="65"/>
+      <c r="I10" s="66" t="s">
+        <v>221</v>
+      </c>
+      <c r="J10" s="67"/>
+      <c r="K10" s="67"/>
+      <c r="L10" s="67"/>
+      <c r="M10" s="80"/>
+      <c r="N10" s="61"/>
+      <c r="O10" s="61"/>
+    </row>
+    <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B11" s="241" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" s="81"/>
+      <c r="D11" s="62">
+        <v>1</v>
+      </c>
+      <c r="E11" s="62">
+        <v>5005</v>
+      </c>
+      <c r="F11" s="63" t="s">
+        <v>191</v>
+      </c>
+      <c r="G11" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="H11" s="65"/>
+      <c r="I11" s="66" t="s">
+        <v>108</v>
+      </c>
+      <c r="J11" s="67" t="s">
+        <v>232</v>
+      </c>
+      <c r="K11" s="67"/>
+      <c r="L11" s="67"/>
+      <c r="M11" s="80"/>
+    </row>
+    <row r="12" spans="1:15" s="182" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B12" s="239" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="124"/>
+      <c r="D12" s="125">
+        <v>1</v>
+      </c>
+      <c r="E12" s="125" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="G12" s="126" t="s">
+        <v>166</v>
+      </c>
+      <c r="H12" s="127"/>
+      <c r="I12" s="128" t="s">
+        <v>207</v>
+      </c>
+      <c r="J12" s="129"/>
+      <c r="K12" s="129"/>
+      <c r="L12" s="129"/>
+      <c r="M12" s="130"/>
+      <c r="N12" s="181"/>
+      <c r="O12" s="181"/>
+    </row>
+    <row r="13" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B13" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="153" t="s">
+        <v>225</v>
+      </c>
+      <c r="D13" s="173">
+        <v>1</v>
+      </c>
+      <c r="E13" s="173" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="174" t="s">
+        <v>193</v>
+      </c>
+      <c r="G13" s="175" t="s">
+        <v>166</v>
+      </c>
+      <c r="H13" s="176"/>
+      <c r="I13" s="177" t="s">
+        <v>126</v>
+      </c>
+      <c r="J13" s="178" t="s">
+        <v>236</v>
+      </c>
+      <c r="K13" s="178"/>
+      <c r="L13" s="178"/>
+      <c r="M13" s="179"/>
+      <c r="N13" s="36"/>
+      <c r="O13" s="36"/>
+    </row>
+    <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B14" s="241" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="145"/>
+      <c r="D14" s="146">
+        <v>12</v>
+      </c>
+      <c r="E14" s="146" t="s">
+        <v>133</v>
+      </c>
+      <c r="F14" s="147" t="s">
+        <v>192</v>
+      </c>
+      <c r="G14" s="148" t="s">
+        <v>166</v>
+      </c>
+      <c r="H14" s="149"/>
+      <c r="I14" s="150" t="s">
+        <v>134</v>
+      </c>
+      <c r="J14" s="151" t="s">
+        <v>231</v>
+      </c>
+      <c r="K14" s="151"/>
+      <c r="L14" s="151"/>
+      <c r="M14" s="152"/>
+      <c r="N14" s="36"/>
+      <c r="O14" s="36"/>
+    </row>
+    <row r="15" spans="1:15" s="194" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B15" s="241" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="145"/>
+      <c r="D15" s="146">
+        <v>1</v>
+      </c>
+      <c r="E15" s="146" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" s="147" t="s">
+        <v>195</v>
+      </c>
+      <c r="G15" s="148" t="s">
+        <v>166</v>
+      </c>
+      <c r="H15" s="149"/>
+      <c r="I15" s="150" t="s">
+        <v>130</v>
+      </c>
+      <c r="J15" s="151" t="s">
+        <v>237</v>
+      </c>
+      <c r="K15" s="151"/>
+      <c r="L15" s="151"/>
+      <c r="M15" s="152"/>
+      <c r="N15" s="193"/>
+      <c r="O15" s="193"/>
+    </row>
+    <row r="16" spans="1:15" s="192" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B16" s="242" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" s="183"/>
+      <c r="D16" s="184">
+        <v>2</v>
+      </c>
+      <c r="E16" s="184" t="s">
+        <v>224</v>
+      </c>
+      <c r="F16" s="185" t="s">
+        <v>222</v>
+      </c>
+      <c r="G16" s="186" t="s">
+        <v>166</v>
+      </c>
+      <c r="H16" s="187"/>
+      <c r="I16" s="188" t="s">
+        <v>223</v>
+      </c>
+      <c r="J16" s="189" t="s">
+        <v>238</v>
+      </c>
+      <c r="K16" s="189"/>
+      <c r="L16" s="189"/>
+      <c r="M16" s="190"/>
+      <c r="N16" s="191"/>
+      <c r="O16" s="191"/>
+    </row>
+    <row r="17" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="116" t="s">
+        <v>185</v>
+      </c>
+      <c r="D17" s="117">
+        <v>1</v>
+      </c>
+      <c r="E17" s="117" t="s">
+        <v>158</v>
+      </c>
+      <c r="F17" s="118" t="s">
+        <v>160</v>
+      </c>
+      <c r="G17" s="119" t="s">
+        <v>167</v>
+      </c>
+      <c r="H17" s="120"/>
+      <c r="I17" s="121" t="s">
+        <v>159</v>
+      </c>
+      <c r="J17" s="236" t="s">
+        <v>235</v>
+      </c>
+      <c r="K17" s="122"/>
+      <c r="L17" s="122"/>
+      <c r="M17" s="123"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="36"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B18" s="241" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" s="82"/>
+      <c r="D18" s="69">
+        <v>1</v>
+      </c>
+      <c r="E18" s="69" t="s">
+        <v>204</v>
+      </c>
+      <c r="F18" s="71" t="s">
+        <v>161</v>
+      </c>
+      <c r="G18" s="72" t="s">
+        <v>168</v>
+      </c>
+      <c r="H18" s="73"/>
+      <c r="I18" s="70" t="s">
+        <v>205</v>
+      </c>
+      <c r="J18" s="235">
+        <v>1210</v>
+      </c>
+      <c r="K18" s="68"/>
+      <c r="L18" s="68"/>
+      <c r="M18" s="83"/>
+      <c r="N18" s="36"/>
+      <c r="O18" s="36"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="82"/>
+      <c r="D19" s="69">
+        <v>1</v>
+      </c>
+      <c r="E19" s="69" t="s">
+        <v>210</v>
+      </c>
+      <c r="F19" s="71" t="s">
+        <v>162</v>
+      </c>
+      <c r="G19" s="72" t="s">
+        <v>169</v>
+      </c>
+      <c r="H19" s="73"/>
+      <c r="I19" s="74" t="s">
+        <v>211</v>
+      </c>
+      <c r="J19" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K19" s="68"/>
+      <c r="L19" s="68"/>
+      <c r="M19" s="83"/>
+      <c r="N19" s="36"/>
+      <c r="O19" s="36"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C20" s="82"/>
+      <c r="D20" s="75">
+        <v>2</v>
+      </c>
+      <c r="E20" s="75" t="s">
+        <v>216</v>
+      </c>
+      <c r="F20" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="G20" s="72" t="s">
+        <v>218</v>
+      </c>
+      <c r="H20" s="77"/>
+      <c r="I20" s="78" t="s">
+        <v>217</v>
+      </c>
+      <c r="J20" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K20" s="68"/>
+      <c r="L20" s="68"/>
+      <c r="M20" s="83"/>
+      <c r="N20" s="36"/>
+      <c r="O20" s="36"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B21" s="241" t="b">
+        <v>1</v>
+      </c>
+      <c r="C21" s="82"/>
+      <c r="D21" s="75">
+        <v>1</v>
+      </c>
+      <c r="E21" s="69" t="s">
+        <v>202</v>
+      </c>
+      <c r="F21" s="76" t="s">
+        <v>163</v>
+      </c>
+      <c r="G21" s="72" t="s">
+        <v>171</v>
+      </c>
+      <c r="H21" s="73"/>
+      <c r="I21" s="74" t="s">
+        <v>201</v>
+      </c>
+      <c r="J21" s="144">
+        <v>2010</v>
+      </c>
+      <c r="K21" s="68"/>
+      <c r="L21" s="68"/>
+      <c r="M21" s="83"/>
+      <c r="N21" s="36"/>
+      <c r="O21" s="36"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C22" s="82"/>
+      <c r="D22" s="75">
+        <v>1</v>
+      </c>
+      <c r="E22" s="69" t="s">
+        <v>214</v>
+      </c>
+      <c r="F22" s="76" t="s">
+        <v>164</v>
+      </c>
+      <c r="G22" s="72" t="s">
+        <v>172</v>
+      </c>
+      <c r="H22" s="73"/>
+      <c r="I22" s="74" t="s">
+        <v>215</v>
+      </c>
+      <c r="J22" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K22" s="68"/>
+      <c r="L22" s="68"/>
+      <c r="M22" s="83"/>
+      <c r="N22" s="36"/>
+      <c r="O22" s="36"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C23" s="82"/>
+      <c r="D23" s="75">
+        <v>2</v>
+      </c>
+      <c r="E23" s="141">
+        <v>560112110017</v>
+      </c>
+      <c r="F23" s="76" t="s">
+        <v>173</v>
+      </c>
+      <c r="G23" s="72">
+        <v>47</v>
+      </c>
+      <c r="H23" s="77"/>
+      <c r="I23" s="78" t="s">
+        <v>203</v>
+      </c>
+      <c r="J23" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K23" s="68"/>
+      <c r="L23" s="68"/>
+      <c r="M23" s="83"/>
+      <c r="N23" s="36"/>
+      <c r="O23" s="36"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="82"/>
+      <c r="D24" s="75">
+        <v>2</v>
+      </c>
+      <c r="E24" s="75" t="s">
+        <v>212</v>
+      </c>
+      <c r="F24" s="76" t="s">
+        <v>174</v>
+      </c>
+      <c r="G24" s="72" t="s">
+        <v>175</v>
+      </c>
+      <c r="H24" s="77"/>
+      <c r="I24" s="78" t="s">
+        <v>213</v>
+      </c>
+      <c r="J24" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K24" s="68"/>
+      <c r="L24" s="68"/>
+      <c r="M24" s="83"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="36"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B25" s="238" t="b">
+        <v>0</v>
+      </c>
+      <c r="C25" s="195"/>
+      <c r="D25" s="196">
+        <v>2</v>
+      </c>
+      <c r="E25" s="196" t="s">
+        <v>197</v>
+      </c>
+      <c r="F25" s="197" t="s">
+        <v>176</v>
+      </c>
+      <c r="G25" s="198" t="s">
+        <v>177</v>
+      </c>
+      <c r="H25" s="199"/>
+      <c r="I25" s="200" t="s">
+        <v>198</v>
+      </c>
+      <c r="J25" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K25" s="202"/>
+      <c r="L25" s="202"/>
+      <c r="M25" s="203"/>
+      <c r="N25" s="36"/>
+      <c r="O25" s="36"/>
+    </row>
+    <row r="26" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="237" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" s="239" t="b">
+        <v>0</v>
+      </c>
+      <c r="C26" s="212"/>
+      <c r="D26" s="213">
+        <v>1</v>
+      </c>
+      <c r="E26" s="213" t="s">
+        <v>199</v>
+      </c>
+      <c r="F26" s="214" t="s">
+        <v>178</v>
+      </c>
+      <c r="G26" s="215" t="s">
+        <v>179</v>
+      </c>
+      <c r="H26" s="216"/>
+      <c r="I26" s="217" t="s">
+        <v>200</v>
+      </c>
+      <c r="J26" s="235" t="s">
+        <v>235</v>
+      </c>
+      <c r="K26" s="219"/>
+      <c r="L26" s="219"/>
+      <c r="M26" s="220"/>
+      <c r="N26" s="108"/>
+      <c r="O26" s="108"/>
+    </row>
+    <row r="27" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B27" s="243" t="b">
+        <v>1</v>
+      </c>
+      <c r="C27" s="204" t="s">
+        <v>226</v>
+      </c>
+      <c r="D27" s="205">
+        <v>1</v>
+      </c>
+      <c r="E27" s="205" t="s">
+        <v>113</v>
+      </c>
+      <c r="F27" s="206" t="s">
+        <v>194</v>
+      </c>
+      <c r="G27" s="207" t="s">
+        <v>166</v>
+      </c>
+      <c r="H27" s="208"/>
+      <c r="I27" s="209" t="s">
+        <v>123</v>
+      </c>
+      <c r="J27" s="210"/>
+      <c r="K27" s="210"/>
+      <c r="L27" s="210"/>
+      <c r="M27" s="211"/>
+      <c r="N27" s="36"/>
+      <c r="O27" s="36"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B28" s="238" t="b">
+        <v>1</v>
+      </c>
+      <c r="C28" s="265"/>
+      <c r="D28" s="266">
+        <v>2</v>
+      </c>
+      <c r="E28" s="266" t="s">
+        <v>101</v>
+      </c>
+      <c r="F28" s="267" t="s">
+        <v>190</v>
+      </c>
+      <c r="G28" s="268" t="s">
+        <v>166</v>
+      </c>
+      <c r="H28" s="269"/>
+      <c r="I28" s="270" t="s">
+        <v>102</v>
+      </c>
+      <c r="J28" s="271"/>
+      <c r="K28" s="271"/>
+      <c r="L28" s="271"/>
+      <c r="M28" s="272"/>
+      <c r="N28" s="36"/>
+      <c r="O28" s="36"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B29" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C29" s="163"/>
+      <c r="D29" s="154"/>
+      <c r="E29" s="154"/>
+      <c r="F29" s="154"/>
+      <c r="G29" s="154"/>
+      <c r="H29" s="154"/>
+      <c r="I29" s="154"/>
+      <c r="J29" s="154"/>
+      <c r="K29" s="154"/>
+      <c r="L29" s="154"/>
+      <c r="M29" s="164"/>
+      <c r="N29" s="36"/>
+      <c r="O29" s="36"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" s="237" t="b">
+        <v>0</v>
+      </c>
+      <c r="B30" s="241" t="b">
+        <v>0</v>
+      </c>
+      <c r="C30" s="163"/>
+      <c r="D30" s="154"/>
+      <c r="E30" s="154"/>
+      <c r="F30" s="154"/>
+      <c r="G30" s="154"/>
+      <c r="H30" s="154"/>
+      <c r="I30" s="154"/>
+      <c r="J30" s="154"/>
+      <c r="K30" s="154"/>
+      <c r="L30" s="154"/>
+      <c r="M30" s="164"/>
+      <c r="N30" s="36"/>
+      <c r="O30" s="36"/>
+    </row>
+    <row r="31" spans="1:15" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="244" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" s="245" t="b">
+        <v>1</v>
+      </c>
+      <c r="C31" s="273"/>
+      <c r="D31" s="274">
+        <v>1</v>
+      </c>
+      <c r="E31" s="274" t="s">
+        <v>119</v>
+      </c>
+      <c r="F31" s="275"/>
+      <c r="G31" s="276" t="s">
+        <v>166</v>
+      </c>
+      <c r="H31" s="277"/>
+      <c r="I31" s="278" t="s">
+        <v>208</v>
+      </c>
+      <c r="J31" s="279"/>
+      <c r="K31" s="279"/>
+      <c r="L31" s="279"/>
+      <c r="M31" s="280"/>
+      <c r="N31" s="61"/>
+      <c r="O31" s="61"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E1:M2"/>
+    <mergeCell ref="E3:M4"/>
+  </mergeCells>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <conditionalFormatting sqref="A6:B31">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>TRUE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10C7034E-99F6-4C64-9A78-788C06E81851}">
   <dimension ref="A1:M32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2679,7 +3939,7 @@
     <col min="8" max="8" width="59.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2690,17 +3950,17 @@
       <c r="B1" s="40">
         <v>1</v>
       </c>
-      <c r="C1" s="149" t="s">
+      <c r="C1" s="228" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="150"/>
-      <c r="E1" s="150"/>
-      <c r="F1" s="150"/>
-      <c r="G1" s="150"/>
-      <c r="H1" s="150"/>
-      <c r="I1" s="150"/>
-      <c r="J1" s="150"/>
-      <c r="K1" s="151"/>
+      <c r="D1" s="229"/>
+      <c r="E1" s="229"/>
+      <c r="F1" s="229"/>
+      <c r="G1" s="229"/>
+      <c r="H1" s="229"/>
+      <c r="I1" s="229"/>
+      <c r="J1" s="229"/>
+      <c r="K1" s="230"/>
       <c r="L1" s="36"/>
       <c r="M1" s="36"/>
     </row>
@@ -2711,15 +3971,15 @@
       <c r="B2" s="40">
         <v>1</v>
       </c>
-      <c r="C2" s="152"/>
-      <c r="D2" s="153"/>
-      <c r="E2" s="153"/>
-      <c r="F2" s="153"/>
-      <c r="G2" s="153"/>
-      <c r="H2" s="153"/>
-      <c r="I2" s="153"/>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154"/>
+      <c r="C2" s="231"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="232"/>
+      <c r="H2" s="232"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="233"/>
       <c r="L2" s="36"/>
       <c r="M2" s="36"/>
     </row>
@@ -2730,105 +3990,107 @@
       <c r="B3" s="40">
         <v>1</v>
       </c>
-      <c r="C3" s="146" t="s">
+      <c r="C3" s="222" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="147"/>
-      <c r="E3" s="147"/>
-      <c r="F3" s="147"/>
-      <c r="G3" s="147"/>
-      <c r="H3" s="147"/>
-      <c r="I3" s="147"/>
-      <c r="J3" s="147"/>
-      <c r="K3" s="148"/>
+      <c r="D3" s="223"/>
+      <c r="E3" s="223"/>
+      <c r="F3" s="223"/>
+      <c r="G3" s="223"/>
+      <c r="H3" s="223"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="224"/>
       <c r="L3" s="36"/>
       <c r="M3" s="36"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="132" t="s">
+      <c r="A4" s="131" t="s">
         <v>140</v>
       </c>
-      <c r="B4" s="133">
+      <c r="B4" s="132">
         <v>46017</v>
       </c>
-      <c r="C4" s="171"/>
-      <c r="D4" s="172"/>
-      <c r="E4" s="172"/>
-      <c r="F4" s="172"/>
-      <c r="G4" s="172"/>
-      <c r="H4" s="172"/>
-      <c r="I4" s="172"/>
-      <c r="J4" s="172"/>
-      <c r="K4" s="173"/>
+      <c r="C4" s="225"/>
+      <c r="D4" s="226"/>
+      <c r="E4" s="226"/>
+      <c r="F4" s="226"/>
+      <c r="G4" s="226"/>
+      <c r="H4" s="226"/>
+      <c r="I4" s="226"/>
+      <c r="J4" s="226"/>
+      <c r="K4" s="227"/>
       <c r="L4" s="36"/>
       <c r="M4" s="36"/>
     </row>
     <row r="5" spans="1:13" s="109" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="174" t="s">
+      <c r="A5" s="159" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="175" t="s">
+      <c r="B5" s="160" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="175" t="s">
+      <c r="C5" s="160" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="175" t="s">
+      <c r="D5" s="160" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="175" t="s">
+      <c r="E5" s="160" t="s">
         <v>165</v>
       </c>
-      <c r="F5" s="175" t="s">
+      <c r="F5" s="160" t="s">
         <v>145</v>
       </c>
-      <c r="G5" s="176" t="s">
+      <c r="G5" s="161" t="s">
         <v>95</v>
       </c>
-      <c r="H5" s="175" t="s">
+      <c r="H5" s="160" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="175" t="s">
+      <c r="I5" s="160" t="s">
         <v>136</v>
       </c>
-      <c r="J5" s="175" t="s">
+      <c r="J5" s="160" t="s">
         <v>137</v>
       </c>
-      <c r="K5" s="177" t="s">
+      <c r="K5" s="162" t="s">
         <v>138</v>
       </c>
       <c r="L5" s="108"/>
       <c r="M5" s="108"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="134" t="s">
+      <c r="A6" s="246" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="135">
-        <v>1</v>
-      </c>
-      <c r="C6" s="135" t="s">
+      <c r="B6" s="134">
+        <v>1</v>
+      </c>
+      <c r="C6" s="134" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="136" t="s">
+      <c r="D6" s="135" t="s">
         <v>186</v>
       </c>
-      <c r="E6" s="137" t="s">
+      <c r="E6" s="136" t="s">
         <v>166</v>
       </c>
-      <c r="F6" s="138"/>
-      <c r="G6" s="139" t="s">
+      <c r="F6" s="137"/>
+      <c r="G6" s="138" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="140"/>
-      <c r="I6" s="140"/>
-      <c r="J6" s="140"/>
-      <c r="K6" s="141"/>
+      <c r="H6" s="139" t="s">
+        <v>229</v>
+      </c>
+      <c r="I6" s="139"/>
+      <c r="J6" s="139"/>
+      <c r="K6" s="140"/>
       <c r="L6" s="36"/>
       <c r="M6" s="36"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="84"/>
+      <c r="A7" s="247"/>
       <c r="B7" s="85">
         <v>1</v>
       </c>
@@ -2845,7 +4107,9 @@
       <c r="G7" s="89" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="90"/>
+      <c r="H7" s="90" t="s">
+        <v>230</v>
+      </c>
       <c r="I7" s="90"/>
       <c r="J7" s="90"/>
       <c r="K7" s="91"/>
@@ -2853,7 +4117,7 @@
       <c r="M7" s="36"/>
     </row>
     <row r="8" spans="1:13" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="100"/>
+      <c r="A8" s="248"/>
       <c r="B8" s="101">
         <v>1</v>
       </c>
@@ -2870,7 +4134,9 @@
       <c r="G8" s="105" t="s">
         <v>104</v>
       </c>
-      <c r="H8" s="106"/>
+      <c r="H8" s="106" t="s">
+        <v>231</v>
+      </c>
       <c r="I8" s="106"/>
       <c r="J8" s="106"/>
       <c r="K8" s="107"/>
@@ -2878,13 +4144,13 @@
       <c r="M8" s="108"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="92" t="s">
+      <c r="A9" s="249" t="s">
         <v>100</v>
       </c>
       <c r="B9" s="93">
         <v>1</v>
       </c>
-      <c r="C9" s="143" t="s">
+      <c r="C9" s="142" t="s">
         <v>206</v>
       </c>
       <c r="D9" s="94" t="s">
@@ -2905,7 +4171,7 @@
       <c r="M9" s="36"/>
     </row>
     <row r="10" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="79"/>
+      <c r="A10" s="250"/>
       <c r="B10" s="62">
         <v>2</v>
       </c>
@@ -2930,7 +4196,7 @@
       <c r="M10" s="61"/>
     </row>
     <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="81"/>
+      <c r="A11" s="251"/>
       <c r="B11" s="62">
         <v>1</v>
       </c>
@@ -2947,194 +4213,204 @@
       <c r="G11" s="66" t="s">
         <v>108</v>
       </c>
-      <c r="H11" s="67"/>
+      <c r="H11" s="67" t="s">
+        <v>232</v>
+      </c>
       <c r="I11" s="67"/>
       <c r="J11" s="67"/>
       <c r="K11" s="80"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="110"/>
-      <c r="B12" s="111">
+      <c r="A12" s="252"/>
+      <c r="B12" s="110">
         <v>2</v>
       </c>
-      <c r="C12" s="111" t="s">
+      <c r="C12" s="110" t="s">
         <v>101</v>
       </c>
-      <c r="D12" s="188" t="s">
+      <c r="D12" s="172" t="s">
         <v>190</v>
       </c>
-      <c r="E12" s="112" t="s">
+      <c r="E12" s="111" t="s">
         <v>166</v>
       </c>
-      <c r="F12" s="113"/>
-      <c r="G12" s="114" t="s">
+      <c r="F12" s="112"/>
+      <c r="G12" s="113" t="s">
         <v>102</v>
       </c>
-      <c r="H12" s="115"/>
-      <c r="I12" s="115"/>
-      <c r="J12" s="115"/>
-      <c r="K12" s="116"/>
+      <c r="H12" s="114"/>
+      <c r="I12" s="114"/>
+      <c r="J12" s="114"/>
+      <c r="K12" s="115"/>
       <c r="L12" s="36"/>
       <c r="M12" s="36"/>
     </row>
-    <row r="13" spans="1:13" s="198" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="125"/>
-      <c r="B13" s="126">
-        <v>1</v>
-      </c>
-      <c r="C13" s="126" t="s">
+    <row r="13" spans="1:13" s="182" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="253"/>
+      <c r="B13" s="125">
+        <v>1</v>
+      </c>
+      <c r="C13" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="196" t="s">
+      <c r="D13" s="180" t="s">
         <v>209</v>
       </c>
-      <c r="E13" s="127" t="s">
+      <c r="E13" s="126" t="s">
         <v>166</v>
       </c>
-      <c r="F13" s="128"/>
-      <c r="G13" s="129" t="s">
+      <c r="F13" s="127"/>
+      <c r="G13" s="128" t="s">
         <v>207</v>
       </c>
-      <c r="H13" s="130"/>
-      <c r="I13" s="130"/>
-      <c r="J13" s="130"/>
-      <c r="K13" s="131"/>
-      <c r="L13" s="197"/>
-      <c r="M13" s="197"/>
+      <c r="H13" s="129"/>
+      <c r="I13" s="129"/>
+      <c r="J13" s="129"/>
+      <c r="K13" s="130"/>
+      <c r="L13" s="181"/>
+      <c r="M13" s="181"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="164" t="s">
+      <c r="A14" s="254" t="s">
         <v>225</v>
       </c>
-      <c r="B14" s="189">
-        <v>1</v>
-      </c>
-      <c r="C14" s="189" t="s">
+      <c r="B14" s="173">
+        <v>1</v>
+      </c>
+      <c r="C14" s="173" t="s">
         <v>110</v>
       </c>
-      <c r="D14" s="190" t="s">
+      <c r="D14" s="174" t="s">
         <v>193</v>
       </c>
-      <c r="E14" s="191" t="s">
+      <c r="E14" s="175" t="s">
         <v>166</v>
       </c>
-      <c r="F14" s="192"/>
-      <c r="G14" s="193" t="s">
+      <c r="F14" s="176"/>
+      <c r="G14" s="177" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="194"/>
-      <c r="I14" s="194"/>
-      <c r="J14" s="194"/>
-      <c r="K14" s="195"/>
+      <c r="H14" s="178" t="s">
+        <v>236</v>
+      </c>
+      <c r="I14" s="178"/>
+      <c r="J14" s="178"/>
+      <c r="K14" s="179"/>
       <c r="L14" s="36"/>
       <c r="M14" s="36"/>
     </row>
     <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="156"/>
-      <c r="B15" s="157">
+      <c r="A15" s="255"/>
+      <c r="B15" s="146">
         <v>12</v>
       </c>
-      <c r="C15" s="157" t="s">
+      <c r="C15" s="146" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="158" t="s">
+      <c r="D15" s="147" t="s">
         <v>192</v>
       </c>
-      <c r="E15" s="159" t="s">
+      <c r="E15" s="148" t="s">
         <v>166</v>
       </c>
-      <c r="F15" s="160"/>
-      <c r="G15" s="161" t="s">
+      <c r="F15" s="149"/>
+      <c r="G15" s="150" t="s">
         <v>134</v>
       </c>
-      <c r="H15" s="162"/>
-      <c r="I15" s="162"/>
-      <c r="J15" s="162"/>
-      <c r="K15" s="163"/>
+      <c r="H15" s="151" t="s">
+        <v>231</v>
+      </c>
+      <c r="I15" s="151"/>
+      <c r="J15" s="151"/>
+      <c r="K15" s="152"/>
       <c r="L15" s="36"/>
       <c r="M15" s="36"/>
     </row>
-    <row r="16" spans="1:13" s="210" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="156"/>
-      <c r="B16" s="157">
-        <v>1</v>
-      </c>
-      <c r="C16" s="157" t="s">
+    <row r="16" spans="1:13" s="194" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="255"/>
+      <c r="B16" s="146">
+        <v>1</v>
+      </c>
+      <c r="C16" s="146" t="s">
         <v>121</v>
       </c>
-      <c r="D16" s="158" t="s">
+      <c r="D16" s="147" t="s">
         <v>195</v>
       </c>
-      <c r="E16" s="159" t="s">
+      <c r="E16" s="148" t="s">
         <v>166</v>
       </c>
-      <c r="F16" s="160"/>
-      <c r="G16" s="161" t="s">
+      <c r="F16" s="149"/>
+      <c r="G16" s="150" t="s">
         <v>130</v>
       </c>
-      <c r="H16" s="162"/>
-      <c r="I16" s="162"/>
-      <c r="J16" s="162"/>
-      <c r="K16" s="163"/>
-      <c r="L16" s="209"/>
-      <c r="M16" s="209"/>
-    </row>
-    <row r="17" spans="1:13" s="208" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="199"/>
-      <c r="B17" s="200">
+      <c r="H16" s="151" t="s">
+        <v>237</v>
+      </c>
+      <c r="I16" s="151"/>
+      <c r="J16" s="151"/>
+      <c r="K16" s="152"/>
+      <c r="L16" s="193"/>
+      <c r="M16" s="193"/>
+    </row>
+    <row r="17" spans="1:13" s="192" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="256"/>
+      <c r="B17" s="184">
         <v>2</v>
       </c>
-      <c r="C17" s="200" t="s">
+      <c r="C17" s="184" t="s">
         <v>224</v>
       </c>
-      <c r="D17" s="201" t="s">
+      <c r="D17" s="185" t="s">
         <v>222</v>
       </c>
-      <c r="E17" s="202" t="s">
+      <c r="E17" s="186" t="s">
         <v>166</v>
       </c>
-      <c r="F17" s="203"/>
-      <c r="G17" s="204" t="s">
+      <c r="F17" s="187"/>
+      <c r="G17" s="188" t="s">
         <v>223</v>
       </c>
-      <c r="H17" s="205"/>
-      <c r="I17" s="205"/>
-      <c r="J17" s="205"/>
-      <c r="K17" s="206"/>
-      <c r="L17" s="207"/>
-      <c r="M17" s="207"/>
+      <c r="H17" s="189" t="s">
+        <v>238</v>
+      </c>
+      <c r="I17" s="189"/>
+      <c r="J17" s="189"/>
+      <c r="K17" s="190"/>
+      <c r="L17" s="191"/>
+      <c r="M17" s="191"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="117" t="s">
+      <c r="A18" s="257" t="s">
         <v>185</v>
       </c>
-      <c r="B18" s="118">
-        <v>1</v>
-      </c>
-      <c r="C18" s="118" t="s">
+      <c r="B18" s="117">
+        <v>1</v>
+      </c>
+      <c r="C18" s="117" t="s">
         <v>158</v>
       </c>
-      <c r="D18" s="119" t="s">
+      <c r="D18" s="118" t="s">
         <v>160</v>
       </c>
-      <c r="E18" s="120" t="s">
+      <c r="E18" s="119" t="s">
         <v>167</v>
       </c>
-      <c r="F18" s="121"/>
-      <c r="G18" s="122" t="s">
+      <c r="F18" s="120"/>
+      <c r="G18" s="121" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="144" t="s">
+      <c r="H18" s="143" t="s">
         <v>183</v>
       </c>
-      <c r="I18" s="123"/>
-      <c r="J18" s="123"/>
-      <c r="K18" s="124"/>
+      <c r="I18" s="122"/>
+      <c r="J18" s="122"/>
+      <c r="K18" s="123"/>
       <c r="L18" s="36"/>
       <c r="M18" s="36"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="82"/>
+      <c r="A19" s="258"/>
       <c r="B19" s="69">
         <v>1</v>
       </c>
@@ -3151,7 +4427,7 @@
       <c r="G19" s="70" t="s">
         <v>205</v>
       </c>
-      <c r="H19" s="145" t="s">
+      <c r="H19" s="144" t="s">
         <v>184</v>
       </c>
       <c r="I19" s="68"/>
@@ -3161,7 +4437,7 @@
       <c r="M19" s="36"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="82"/>
+      <c r="A20" s="258"/>
       <c r="B20" s="69">
         <v>1</v>
       </c>
@@ -3178,7 +4454,7 @@
       <c r="G20" s="74" t="s">
         <v>211</v>
       </c>
-      <c r="H20" s="145" t="s">
+      <c r="H20" s="144" t="s">
         <v>219</v>
       </c>
       <c r="I20" s="68"/>
@@ -3188,7 +4464,7 @@
       <c r="M20" s="36"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="82"/>
+      <c r="A21" s="258"/>
       <c r="B21" s="75">
         <v>2</v>
       </c>
@@ -3205,7 +4481,7 @@
       <c r="G21" s="78" t="s">
         <v>217</v>
       </c>
-      <c r="H21" s="145" t="s">
+      <c r="H21" s="144" t="s">
         <v>182</v>
       </c>
       <c r="I21" s="68"/>
@@ -3215,7 +4491,7 @@
       <c r="M21" s="36"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="82"/>
+      <c r="A22" s="258"/>
       <c r="B22" s="75">
         <v>1</v>
       </c>
@@ -3232,7 +4508,7 @@
       <c r="G22" s="74" t="s">
         <v>201</v>
       </c>
-      <c r="H22" s="145" t="s">
+      <c r="H22" s="144" t="s">
         <v>181</v>
       </c>
       <c r="I22" s="68"/>
@@ -3242,7 +4518,7 @@
       <c r="M22" s="36"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="82"/>
+      <c r="A23" s="258"/>
       <c r="B23" s="75">
         <v>1</v>
       </c>
@@ -3259,7 +4535,7 @@
       <c r="G23" s="74" t="s">
         <v>215</v>
       </c>
-      <c r="H23" s="145" t="s">
+      <c r="H23" s="144" t="s">
         <v>180</v>
       </c>
       <c r="I23" s="68"/>
@@ -3269,11 +4545,11 @@
       <c r="M23" s="36"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="82"/>
+      <c r="A24" s="258"/>
       <c r="B24" s="75">
         <v>2</v>
       </c>
-      <c r="C24" s="142">
+      <c r="C24" s="141">
         <v>560112110017</v>
       </c>
       <c r="D24" s="76" t="s">
@@ -3286,7 +4562,7 @@
       <c r="G24" s="78" t="s">
         <v>203</v>
       </c>
-      <c r="H24" s="145" t="s">
+      <c r="H24" s="144" t="s">
         <v>180</v>
       </c>
       <c r="I24" s="68"/>
@@ -3296,7 +4572,7 @@
       <c r="M24" s="36"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="82"/>
+      <c r="A25" s="258"/>
       <c r="B25" s="75">
         <v>2</v>
       </c>
@@ -3313,7 +4589,7 @@
       <c r="G25" s="78" t="s">
         <v>213</v>
       </c>
-      <c r="H25" s="145" t="s">
+      <c r="H25" s="144" t="s">
         <v>182</v>
       </c>
       <c r="I25" s="68"/>
@@ -3323,151 +4599,151 @@
       <c r="M25" s="36"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="211"/>
-      <c r="B26" s="212">
+      <c r="A26" s="259"/>
+      <c r="B26" s="196">
         <v>2</v>
       </c>
-      <c r="C26" s="212" t="s">
+      <c r="C26" s="196" t="s">
         <v>197</v>
       </c>
-      <c r="D26" s="213" t="s">
+      <c r="D26" s="197" t="s">
         <v>176</v>
       </c>
-      <c r="E26" s="214" t="s">
+      <c r="E26" s="198" t="s">
         <v>177</v>
       </c>
-      <c r="F26" s="215"/>
-      <c r="G26" s="216" t="s">
+      <c r="F26" s="199"/>
+      <c r="G26" s="200" t="s">
         <v>198</v>
       </c>
-      <c r="H26" s="217" t="s">
+      <c r="H26" s="201" t="s">
         <v>182</v>
       </c>
-      <c r="I26" s="218"/>
-      <c r="J26" s="218"/>
-      <c r="K26" s="219"/>
+      <c r="I26" s="202"/>
+      <c r="J26" s="202"/>
+      <c r="K26" s="203"/>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
     </row>
     <row r="27" spans="1:13" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="228"/>
-      <c r="B27" s="229">
-        <v>1</v>
-      </c>
-      <c r="C27" s="229" t="s">
+      <c r="A27" s="260"/>
+      <c r="B27" s="213">
+        <v>1</v>
+      </c>
+      <c r="C27" s="213" t="s">
         <v>199</v>
       </c>
-      <c r="D27" s="230" t="s">
+      <c r="D27" s="214" t="s">
         <v>178</v>
       </c>
-      <c r="E27" s="231" t="s">
+      <c r="E27" s="215" t="s">
         <v>179</v>
       </c>
-      <c r="F27" s="232"/>
-      <c r="G27" s="233" t="s">
+      <c r="F27" s="216"/>
+      <c r="G27" s="217" t="s">
         <v>200</v>
       </c>
-      <c r="H27" s="234" t="s">
+      <c r="H27" s="218" t="s">
         <v>180</v>
       </c>
-      <c r="I27" s="235"/>
-      <c r="J27" s="235"/>
-      <c r="K27" s="236"/>
+      <c r="I27" s="219"/>
+      <c r="J27" s="219"/>
+      <c r="K27" s="220"/>
       <c r="L27" s="108"/>
       <c r="M27" s="108"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="220" t="s">
+      <c r="A28" s="261" t="s">
         <v>226</v>
       </c>
-      <c r="B28" s="221">
-        <v>1</v>
-      </c>
-      <c r="C28" s="221" t="s">
+      <c r="B28" s="205">
+        <v>1</v>
+      </c>
+      <c r="C28" s="205" t="s">
         <v>113</v>
       </c>
-      <c r="D28" s="222" t="s">
+      <c r="D28" s="206" t="s">
         <v>194</v>
       </c>
-      <c r="E28" s="223" t="s">
+      <c r="E28" s="207" t="s">
         <v>166</v>
       </c>
-      <c r="F28" s="224"/>
-      <c r="G28" s="225" t="s">
+      <c r="F28" s="208"/>
+      <c r="G28" s="209" t="s">
         <v>123</v>
       </c>
-      <c r="H28" s="226"/>
-      <c r="I28" s="226"/>
-      <c r="J28" s="226"/>
-      <c r="K28" s="227"/>
+      <c r="H28" s="210"/>
+      <c r="I28" s="210"/>
+      <c r="J28" s="210"/>
+      <c r="K28" s="211"/>
       <c r="L28" s="36"/>
       <c r="M28" s="36"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="178"/>
-      <c r="B29" s="166"/>
-      <c r="C29" s="167"/>
-      <c r="D29" s="168"/>
-      <c r="E29" s="165"/>
-      <c r="F29" s="169"/>
-      <c r="G29" s="170"/>
-      <c r="H29" s="165"/>
-      <c r="I29" s="165"/>
-      <c r="J29" s="165"/>
-      <c r="K29" s="179"/>
+      <c r="A29" s="262"/>
+      <c r="B29" s="263"/>
+      <c r="C29" s="155"/>
+      <c r="D29" s="156"/>
+      <c r="E29" s="154"/>
+      <c r="F29" s="157"/>
+      <c r="G29" s="158"/>
+      <c r="H29" s="154"/>
+      <c r="I29" s="154"/>
+      <c r="J29" s="154"/>
+      <c r="K29" s="164"/>
       <c r="L29" s="36"/>
       <c r="M29" s="36"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="178"/>
-      <c r="B30" s="165"/>
-      <c r="C30" s="165"/>
-      <c r="D30" s="165"/>
-      <c r="E30" s="165"/>
-      <c r="F30" s="165"/>
-      <c r="G30" s="165"/>
-      <c r="H30" s="165"/>
-      <c r="I30" s="165"/>
-      <c r="J30" s="165"/>
-      <c r="K30" s="179"/>
+      <c r="A30" s="262"/>
+      <c r="B30" s="263"/>
+      <c r="C30" s="154"/>
+      <c r="D30" s="154"/>
+      <c r="E30" s="154"/>
+      <c r="F30" s="154"/>
+      <c r="G30" s="154"/>
+      <c r="H30" s="154"/>
+      <c r="I30" s="154"/>
+      <c r="J30" s="154"/>
+      <c r="K30" s="164"/>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="178"/>
-      <c r="B31" s="165"/>
-      <c r="C31" s="165"/>
-      <c r="D31" s="165"/>
-      <c r="E31" s="165"/>
-      <c r="F31" s="165"/>
-      <c r="G31" s="165"/>
-      <c r="H31" s="165"/>
-      <c r="I31" s="165"/>
-      <c r="J31" s="165"/>
-      <c r="K31" s="179"/>
+      <c r="A31" s="262"/>
+      <c r="B31" s="263"/>
+      <c r="C31" s="154"/>
+      <c r="D31" s="154"/>
+      <c r="E31" s="154"/>
+      <c r="F31" s="154"/>
+      <c r="G31" s="154"/>
+      <c r="H31" s="154"/>
+      <c r="I31" s="154"/>
+      <c r="J31" s="154"/>
+      <c r="K31" s="164"/>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
     </row>
     <row r="32" spans="1:13" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="180"/>
-      <c r="B32" s="181">
-        <v>1</v>
-      </c>
-      <c r="C32" s="181" t="s">
+      <c r="A32" s="264"/>
+      <c r="B32" s="165">
+        <v>1</v>
+      </c>
+      <c r="C32" s="165" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="182"/>
-      <c r="E32" s="183" t="s">
+      <c r="D32" s="166"/>
+      <c r="E32" s="167" t="s">
         <v>166</v>
       </c>
-      <c r="F32" s="184"/>
-      <c r="G32" s="185" t="s">
+      <c r="F32" s="168"/>
+      <c r="G32" s="169" t="s">
         <v>208</v>
       </c>
-      <c r="H32" s="186"/>
-      <c r="I32" s="186"/>
-      <c r="J32" s="186"/>
-      <c r="K32" s="187"/>
+      <c r="H32" s="170"/>
+      <c r="I32" s="170"/>
+      <c r="J32" s="170"/>
+      <c r="K32" s="171"/>
       <c r="L32" s="61"/>
       <c r="M32" s="61"/>
     </row>
@@ -3480,7 +4756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:L65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3503,14 +4779,14 @@
       <c r="E2" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="155" t="s">
+      <c r="F2" s="234" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="155"/>
-      <c r="K2" s="155"/>
+      <c r="G2" s="234"/>
+      <c r="H2" s="234"/>
+      <c r="I2" s="234"/>
+      <c r="J2" s="234"/>
+      <c r="K2" s="234"/>
       <c r="L2" s="59" t="s">
         <v>149</v>
       </c>
@@ -4061,7 +5337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EEC52D2-7558-455D-94BF-A1AB4EDE4282}">
   <dimension ref="B2:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4164,16 +5440,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB492BA-2F79-49D5-B025-264C23C3C544}">
-  <dimension ref="B3:H26"/>
+  <dimension ref="B3:H24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="34">
         <v>12</v>
       </c>
@@ -4186,7 +5462,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="34">
         <v>1</v>
       </c>
@@ -4199,12 +5475,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C5" s="37" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="36" t="s">
         <v>109</v>
       </c>
@@ -4212,7 +5488,7 @@
         <v>3825</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C8" s="34">
         <v>10</v>
       </c>
@@ -4225,17 +5501,38 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="19" spans="4:8" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D12" s="34">
+        <v>12</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="35" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="3:8" ht="23.25" x14ac:dyDescent="0.35">
       <c r="D19" s="42" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="20" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D20" s="34">
         <v>1</v>
       </c>
@@ -4248,7 +5545,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="21" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D21" s="34">
         <v>1</v>
       </c>
@@ -4261,7 +5558,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="22" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D22" s="34">
         <v>2</v>
       </c>
@@ -4274,38 +5571,29 @@
         <v>122</v>
       </c>
     </row>
-    <row r="23" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D23" t="s">
-        <v>148</v>
-      </c>
-      <c r="E23" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D25" s="34">
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D23" s="34">
         <v>12</v>
       </c>
-      <c r="E25" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="35" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="26" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D26" s="34">
-        <v>12</v>
-      </c>
-      <c r="E26" s="34" t="s">
+      <c r="E23" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="35" t="s">
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="35" t="s">
         <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C24" s="221"/>
+      <c r="D24" s="34">
+        <v>100</v>
+      </c>
+      <c r="E24" s="34" t="s">
+        <v>227</v>
+      </c>
+      <c r="H24" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
p much done, no nixie hat board though
</commit_message>
<xml_diff>
--- a/Documents/OMNIXIE_sheets.xlsx
+++ b/Documents/OMNIXIE_sheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21nic\OneDrive\Desktop\NIXIE\OMNIXIE\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E1B675-60BB-46F2-B3B3-C2EC7950E151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADE8EB2-ADF0-49D9-87D9-7E859E73AA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="243">
   <si>
     <t>A: ADC, A7 (ADC_IN7)</t>
   </si>
@@ -760,6 +760,15 @@
   </si>
   <si>
     <t>J1,J6</t>
+  </si>
+  <si>
+    <t>_0603</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>R10,R16</t>
   </si>
 </sst>
 </file>
@@ -1634,7 +1643,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="281">
+  <cellXfs count="279">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2144,64 +2153,7 @@
     <xf numFmtId="0" fontId="7" fillId="16" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2209,7 +2161,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2217,7 +2169,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2225,7 +2177,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2233,7 +2185,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2241,7 +2193,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2249,7 +2201,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2257,7 +2209,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2265,7 +2217,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -2366,6 +2318,57 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2373,7 +2376,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="3" xr:uid="{B93126DE-0D01-4C50-8056-E448E7756006}"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -2388,13 +2391,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2928,7 +2924,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE706952-430C-44AA-84E6-C88695E38A9F}">
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
@@ -2939,7 +2935,7 @@
     <col min="7" max="7" width="9.85546875" customWidth="1"/>
     <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="121.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="72.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6.140625" bestFit="1" customWidth="1"/>
@@ -2955,17 +2951,17 @@
       <c r="D1" s="40">
         <v>1</v>
       </c>
-      <c r="E1" s="228" t="s">
+      <c r="E1" s="266" t="s">
         <v>139</v>
       </c>
-      <c r="F1" s="229"/>
-      <c r="G1" s="229"/>
-      <c r="H1" s="229"/>
-      <c r="I1" s="229"/>
-      <c r="J1" s="229"/>
-      <c r="K1" s="229"/>
-      <c r="L1" s="229"/>
-      <c r="M1" s="230"/>
+      <c r="F1" s="267"/>
+      <c r="G1" s="267"/>
+      <c r="H1" s="267"/>
+      <c r="I1" s="267"/>
+      <c r="J1" s="267"/>
+      <c r="K1" s="267"/>
+      <c r="L1" s="267"/>
+      <c r="M1" s="268"/>
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
@@ -2978,15 +2974,15 @@
       <c r="D2" s="40">
         <v>1</v>
       </c>
-      <c r="E2" s="231"/>
-      <c r="F2" s="232"/>
-      <c r="G2" s="232"/>
-      <c r="H2" s="232"/>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
-      <c r="M2" s="233"/>
+      <c r="E2" s="269"/>
+      <c r="F2" s="270"/>
+      <c r="G2" s="270"/>
+      <c r="H2" s="270"/>
+      <c r="I2" s="270"/>
+      <c r="J2" s="270"/>
+      <c r="K2" s="270"/>
+      <c r="L2" s="270"/>
+      <c r="M2" s="271"/>
       <c r="N2" s="36"/>
       <c r="O2" s="36"/>
     </row>
@@ -2999,17 +2995,17 @@
       <c r="D3" s="40">
         <v>1</v>
       </c>
-      <c r="E3" s="222" t="s">
+      <c r="E3" s="272" t="s">
         <v>141</v>
       </c>
-      <c r="F3" s="223"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="223"/>
-      <c r="I3" s="223"/>
-      <c r="J3" s="223"/>
-      <c r="K3" s="223"/>
-      <c r="L3" s="223"/>
-      <c r="M3" s="224"/>
+      <c r="F3" s="273"/>
+      <c r="G3" s="273"/>
+      <c r="H3" s="273"/>
+      <c r="I3" s="273"/>
+      <c r="J3" s="273"/>
+      <c r="K3" s="273"/>
+      <c r="L3" s="273"/>
+      <c r="M3" s="274"/>
       <c r="N3" s="36"/>
       <c r="O3" s="36"/>
     </row>
@@ -3022,15 +3018,15 @@
       <c r="D4" s="132">
         <v>46017</v>
       </c>
-      <c r="E4" s="225"/>
-      <c r="F4" s="226"/>
-      <c r="G4" s="226"/>
-      <c r="H4" s="226"/>
-      <c r="I4" s="226"/>
-      <c r="J4" s="226"/>
-      <c r="K4" s="226"/>
-      <c r="L4" s="226"/>
-      <c r="M4" s="227"/>
+      <c r="E4" s="275"/>
+      <c r="F4" s="276"/>
+      <c r="G4" s="276"/>
+      <c r="H4" s="276"/>
+      <c r="I4" s="276"/>
+      <c r="J4" s="276"/>
+      <c r="K4" s="276"/>
+      <c r="L4" s="276"/>
+      <c r="M4" s="277"/>
       <c r="N4" s="36"/>
       <c r="O4" s="36"/>
     </row>
@@ -3078,10 +3074,10 @@
       <c r="O5" s="108"/>
     </row>
     <row r="6" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="237" t="b">
+      <c r="A6" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B6" s="237" t="b">
+      <c r="B6" s="222" t="b">
         <v>1</v>
       </c>
       <c r="C6" s="133" t="s">
@@ -3113,10 +3109,10 @@
       <c r="O6" s="36"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="237" t="b">
+      <c r="A7" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B7" s="238" t="b">
+      <c r="B7" s="223" t="b">
         <v>1</v>
       </c>
       <c r="C7" s="84"/>
@@ -3146,10 +3142,10 @@
       <c r="O7" s="36"/>
     </row>
     <row r="8" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="237" t="b">
+      <c r="A8" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B8" s="239" t="b">
+      <c r="B8" s="224" t="b">
         <v>1</v>
       </c>
       <c r="C8" s="100"/>
@@ -3179,10 +3175,10 @@
       <c r="O8" s="108"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="237" t="b">
+      <c r="A9" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B9" s="237" t="b">
+      <c r="B9" s="222" t="b">
         <v>1</v>
       </c>
       <c r="C9" s="92" t="s">
@@ -3212,10 +3208,10 @@
       <c r="O9" s="36"/>
     </row>
     <row r="10" spans="1:15" s="60" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="240" t="b">
+      <c r="A10" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="225" t="b">
         <v>0</v>
       </c>
       <c r="C10" s="79"/>
@@ -3243,15 +3239,15 @@
       <c r="O10" s="61"/>
     </row>
     <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="237" t="b">
+      <c r="A11" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B11" s="241" t="b">
+      <c r="B11" s="226" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="81"/>
       <c r="D11" s="62">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E11" s="62">
         <v>5005</v>
@@ -3274,10 +3270,10 @@
       <c r="M11" s="80"/>
     </row>
     <row r="12" spans="1:15" s="182" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="237" t="b">
+      <c r="A12" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B12" s="239" t="b">
+      <c r="B12" s="224" t="b">
         <v>1</v>
       </c>
       <c r="C12" s="124"/>
@@ -3305,10 +3301,10 @@
       <c r="O12" s="181"/>
     </row>
     <row r="13" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="237" t="b">
+      <c r="A13" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B13" s="237" t="b">
+      <c r="B13" s="222" t="b">
         <v>1</v>
       </c>
       <c r="C13" s="153" t="s">
@@ -3340,10 +3336,10 @@
       <c r="O13" s="36"/>
     </row>
     <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="237" t="b">
+      <c r="A14" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B14" s="241" t="b">
+      <c r="B14" s="226" t="b">
         <v>1</v>
       </c>
       <c r="C14" s="145"/>
@@ -3373,10 +3369,10 @@
       <c r="O14" s="36"/>
     </row>
     <row r="15" spans="1:15" s="194" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="237" t="b">
+      <c r="A15" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B15" s="241" t="b">
+      <c r="B15" s="226" t="b">
         <v>1</v>
       </c>
       <c r="C15" s="145"/>
@@ -3406,10 +3402,10 @@
       <c r="O15" s="193"/>
     </row>
     <row r="16" spans="1:15" s="192" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="237" t="b">
+      <c r="A16" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B16" s="242" t="b">
+      <c r="B16" s="227" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="183"/>
@@ -3439,10 +3435,10 @@
       <c r="O16" s="191"/>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" s="237" t="b">
+      <c r="A17" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="222" t="b">
         <v>0</v>
       </c>
       <c r="C17" s="116" t="s">
@@ -3464,7 +3460,7 @@
       <c r="I17" s="121" t="s">
         <v>159</v>
       </c>
-      <c r="J17" s="236" t="s">
+      <c r="J17" s="143" t="s">
         <v>235</v>
       </c>
       <c r="K17" s="122"/>
@@ -3474,10 +3470,10 @@
       <c r="O17" s="36"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="237" t="b">
+      <c r="A18" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B18" s="241" t="b">
+      <c r="B18" s="226" t="b">
         <v>1</v>
       </c>
       <c r="C18" s="82"/>
@@ -3497,7 +3493,7 @@
       <c r="I18" s="70" t="s">
         <v>205</v>
       </c>
-      <c r="J18" s="235">
+      <c r="J18" s="144">
         <v>1210</v>
       </c>
       <c r="K18" s="68"/>
@@ -3507,15 +3503,15 @@
       <c r="O18" s="36"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B19" s="241" t="b">
+      <c r="A19" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="226" t="b">
         <v>0</v>
       </c>
       <c r="C19" s="82"/>
       <c r="D19" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E19" s="69" t="s">
         <v>210</v>
@@ -3530,7 +3526,7 @@
       <c r="I19" s="74" t="s">
         <v>211</v>
       </c>
-      <c r="J19" s="235" t="s">
+      <c r="J19" s="144" t="s">
         <v>235</v>
       </c>
       <c r="K19" s="68"/>
@@ -3540,11 +3536,11 @@
       <c r="O19" s="36"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B20" s="241" t="b">
+      <c r="A20" s="222" t="b">
         <v>0</v>
+      </c>
+      <c r="B20" s="226" t="b">
+        <v>1</v>
       </c>
       <c r="C20" s="82"/>
       <c r="D20" s="75">
@@ -3563,8 +3559,8 @@
       <c r="I20" s="78" t="s">
         <v>217</v>
       </c>
-      <c r="J20" s="235" t="s">
-        <v>235</v>
+      <c r="J20" s="144" t="s">
+        <v>240</v>
       </c>
       <c r="K20" s="68"/>
       <c r="L20" s="68"/>
@@ -3573,31 +3569,31 @@
       <c r="O20" s="36"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="237" t="b">
+      <c r="A21" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B21" s="241" t="b">
-        <v>1</v>
+      <c r="B21" s="226" t="b">
+        <v>0</v>
       </c>
       <c r="C21" s="82"/>
       <c r="D21" s="75">
-        <v>1</v>
-      </c>
-      <c r="E21" s="69" t="s">
-        <v>202</v>
+        <v>2</v>
+      </c>
+      <c r="E21" s="75" t="s">
+        <v>166</v>
       </c>
       <c r="F21" s="76" t="s">
-        <v>163</v>
+        <v>242</v>
       </c>
       <c r="G21" s="72" t="s">
-        <v>171</v>
-      </c>
-      <c r="H21" s="73"/>
-      <c r="I21" s="74" t="s">
-        <v>201</v>
-      </c>
-      <c r="J21" s="144">
-        <v>2010</v>
+        <v>241</v>
+      </c>
+      <c r="H21" s="77"/>
+      <c r="I21" s="78" t="s">
+        <v>166</v>
+      </c>
+      <c r="J21" s="144" t="s">
+        <v>235</v>
       </c>
       <c r="K21" s="68"/>
       <c r="L21" s="68"/>
@@ -3606,31 +3602,31 @@
       <c r="O21" s="36"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B22" s="241" t="b">
+      <c r="A22" s="222" t="b">
         <v>0</v>
+      </c>
+      <c r="B22" s="226" t="b">
+        <v>1</v>
       </c>
       <c r="C22" s="82"/>
       <c r="D22" s="75">
         <v>1</v>
       </c>
       <c r="E22" s="69" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="F22" s="76" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G22" s="72" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H22" s="73"/>
       <c r="I22" s="74" t="s">
-        <v>215</v>
-      </c>
-      <c r="J22" s="235" t="s">
-        <v>235</v>
+        <v>201</v>
+      </c>
+      <c r="J22" s="144">
+        <v>2010</v>
       </c>
       <c r="K22" s="68"/>
       <c r="L22" s="68"/>
@@ -3639,30 +3635,30 @@
       <c r="O22" s="36"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B23" s="241" t="b">
+      <c r="A23" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" s="226" t="b">
         <v>0</v>
       </c>
       <c r="C23" s="82"/>
       <c r="D23" s="75">
-        <v>2</v>
-      </c>
-      <c r="E23" s="141">
-        <v>560112110017</v>
+        <v>1</v>
+      </c>
+      <c r="E23" s="69" t="s">
+        <v>214</v>
       </c>
       <c r="F23" s="76" t="s">
-        <v>173</v>
-      </c>
-      <c r="G23" s="72">
-        <v>47</v>
-      </c>
-      <c r="H23" s="77"/>
-      <c r="I23" s="78" t="s">
-        <v>203</v>
-      </c>
-      <c r="J23" s="235" t="s">
+        <v>164</v>
+      </c>
+      <c r="G23" s="72" t="s">
+        <v>172</v>
+      </c>
+      <c r="H23" s="73"/>
+      <c r="I23" s="74" t="s">
+        <v>215</v>
+      </c>
+      <c r="J23" s="144" t="s">
         <v>235</v>
       </c>
       <c r="K23" s="68"/>
@@ -3672,30 +3668,30 @@
       <c r="O23" s="36"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B24" s="241" t="b">
+      <c r="A24" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="226" t="b">
         <v>0</v>
       </c>
       <c r="C24" s="82"/>
       <c r="D24" s="75">
         <v>2</v>
       </c>
-      <c r="E24" s="75" t="s">
-        <v>212</v>
+      <c r="E24" s="141">
+        <v>560112110017</v>
       </c>
       <c r="F24" s="76" t="s">
-        <v>174</v>
-      </c>
-      <c r="G24" s="72" t="s">
-        <v>175</v>
+        <v>173</v>
+      </c>
+      <c r="G24" s="72">
+        <v>47</v>
       </c>
       <c r="H24" s="77"/>
       <c r="I24" s="78" t="s">
-        <v>213</v>
-      </c>
-      <c r="J24" s="235" t="s">
+        <v>203</v>
+      </c>
+      <c r="J24" s="144" t="s">
         <v>235</v>
       </c>
       <c r="K24" s="68"/>
@@ -3705,161 +3701,173 @@
       <c r="O24" s="36"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B25" s="238" t="b">
+      <c r="A25" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B25" s="226" t="b">
         <v>0</v>
       </c>
-      <c r="C25" s="195"/>
-      <c r="D25" s="196">
+      <c r="C25" s="82"/>
+      <c r="D25" s="75">
         <v>2</v>
       </c>
-      <c r="E25" s="196" t="s">
-        <v>197</v>
-      </c>
-      <c r="F25" s="197" t="s">
-        <v>176</v>
-      </c>
-      <c r="G25" s="198" t="s">
-        <v>177</v>
-      </c>
-      <c r="H25" s="199"/>
-      <c r="I25" s="200" t="s">
-        <v>198</v>
-      </c>
-      <c r="J25" s="235" t="s">
+      <c r="E25" s="75" t="s">
+        <v>212</v>
+      </c>
+      <c r="F25" s="76" t="s">
+        <v>174</v>
+      </c>
+      <c r="G25" s="72" t="s">
+        <v>175</v>
+      </c>
+      <c r="H25" s="77"/>
+      <c r="I25" s="78" t="s">
+        <v>213</v>
+      </c>
+      <c r="J25" s="144" t="s">
         <v>235</v>
       </c>
-      <c r="K25" s="202"/>
-      <c r="L25" s="202"/>
-      <c r="M25" s="203"/>
+      <c r="K25" s="68"/>
+      <c r="L25" s="68"/>
+      <c r="M25" s="83"/>
       <c r="N25" s="36"/>
       <c r="O25" s="36"/>
     </row>
-    <row r="26" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="237" t="b">
-        <v>1</v>
-      </c>
-      <c r="B26" s="239" t="b">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" s="223" t="b">
         <v>0</v>
       </c>
-      <c r="C26" s="212"/>
-      <c r="D26" s="213">
-        <v>1</v>
-      </c>
-      <c r="E26" s="213" t="s">
+      <c r="C26" s="195"/>
+      <c r="D26" s="196">
+        <v>2</v>
+      </c>
+      <c r="E26" s="196" t="s">
+        <v>197</v>
+      </c>
+      <c r="F26" s="197" t="s">
+        <v>176</v>
+      </c>
+      <c r="G26" s="198" t="s">
+        <v>177</v>
+      </c>
+      <c r="H26" s="199"/>
+      <c r="I26" s="200" t="s">
+        <v>198</v>
+      </c>
+      <c r="J26" s="144" t="s">
+        <v>235</v>
+      </c>
+      <c r="K26" s="202"/>
+      <c r="L26" s="202"/>
+      <c r="M26" s="203"/>
+      <c r="N26" s="36"/>
+      <c r="O26" s="36"/>
+    </row>
+    <row r="27" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" s="224" t="b">
+        <v>0</v>
+      </c>
+      <c r="C27" s="212"/>
+      <c r="D27" s="213">
+        <v>1</v>
+      </c>
+      <c r="E27" s="213" t="s">
         <v>199</v>
       </c>
-      <c r="F26" s="214" t="s">
+      <c r="F27" s="214" t="s">
         <v>178</v>
       </c>
-      <c r="G26" s="215" t="s">
+      <c r="G27" s="215" t="s">
         <v>179</v>
       </c>
-      <c r="H26" s="216"/>
-      <c r="I26" s="217" t="s">
+      <c r="H27" s="216"/>
+      <c r="I27" s="217" t="s">
         <v>200</v>
       </c>
-      <c r="J26" s="235" t="s">
+      <c r="J27" s="144" t="s">
         <v>235</v>
       </c>
-      <c r="K26" s="219"/>
-      <c r="L26" s="219"/>
-      <c r="M26" s="220"/>
-      <c r="N26" s="108"/>
-      <c r="O26" s="108"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="237" t="b">
+      <c r="K27" s="219"/>
+      <c r="L27" s="219"/>
+      <c r="M27" s="220"/>
+      <c r="N27" s="108"/>
+      <c r="O27" s="108"/>
+    </row>
+    <row r="28" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B27" s="243" t="b">
-        <v>1</v>
-      </c>
-      <c r="C27" s="204" t="s">
+      <c r="B28" s="228" t="b">
+        <v>1</v>
+      </c>
+      <c r="C28" s="204" t="s">
         <v>226</v>
       </c>
-      <c r="D27" s="205">
-        <v>1</v>
-      </c>
-      <c r="E27" s="205" t="s">
+      <c r="D28" s="205">
+        <v>1</v>
+      </c>
+      <c r="E28" s="205" t="s">
         <v>113</v>
       </c>
-      <c r="F27" s="206" t="s">
+      <c r="F28" s="206" t="s">
         <v>194</v>
       </c>
-      <c r="G27" s="207" t="s">
+      <c r="G28" s="207" t="s">
         <v>166</v>
       </c>
-      <c r="H27" s="208"/>
-      <c r="I27" s="209" t="s">
+      <c r="H28" s="208"/>
+      <c r="I28" s="209" t="s">
         <v>123</v>
       </c>
-      <c r="J27" s="210"/>
-      <c r="K27" s="210"/>
-      <c r="L27" s="210"/>
-      <c r="M27" s="211"/>
-      <c r="N27" s="36"/>
-      <c r="O27" s="36"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="237" t="b">
-        <v>0</v>
-      </c>
-      <c r="B28" s="238" t="b">
-        <v>1</v>
-      </c>
-      <c r="C28" s="265"/>
-      <c r="D28" s="266">
-        <v>2</v>
-      </c>
-      <c r="E28" s="266" t="s">
-        <v>101</v>
-      </c>
-      <c r="F28" s="267" t="s">
-        <v>190</v>
-      </c>
-      <c r="G28" s="268" t="s">
-        <v>166</v>
-      </c>
-      <c r="H28" s="269"/>
-      <c r="I28" s="270" t="s">
-        <v>102</v>
-      </c>
-      <c r="J28" s="271"/>
-      <c r="K28" s="271"/>
-      <c r="L28" s="271"/>
-      <c r="M28" s="272"/>
+      <c r="J28" s="210"/>
+      <c r="K28" s="210"/>
+      <c r="L28" s="210"/>
+      <c r="M28" s="211"/>
       <c r="N28" s="36"/>
       <c r="O28" s="36"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="237" t="b">
+      <c r="A29" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B29" s="241" t="b">
-        <v>0</v>
-      </c>
-      <c r="C29" s="163"/>
-      <c r="D29" s="154"/>
-      <c r="E29" s="154"/>
-      <c r="F29" s="154"/>
-      <c r="G29" s="154"/>
-      <c r="H29" s="154"/>
-      <c r="I29" s="154"/>
-      <c r="J29" s="154"/>
-      <c r="K29" s="154"/>
-      <c r="L29" s="154"/>
-      <c r="M29" s="164"/>
+      <c r="B29" s="223" t="b">
+        <v>1</v>
+      </c>
+      <c r="C29" s="250"/>
+      <c r="D29" s="251">
+        <v>2</v>
+      </c>
+      <c r="E29" s="251" t="s">
+        <v>101</v>
+      </c>
+      <c r="F29" s="252" t="s">
+        <v>190</v>
+      </c>
+      <c r="G29" s="253" t="s">
+        <v>166</v>
+      </c>
+      <c r="H29" s="254"/>
+      <c r="I29" s="255" t="s">
+        <v>102</v>
+      </c>
+      <c r="J29" s="256"/>
+      <c r="K29" s="256"/>
+      <c r="L29" s="256"/>
+      <c r="M29" s="257"/>
       <c r="N29" s="36"/>
       <c r="O29" s="36"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="237" t="b">
+      <c r="A30" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B30" s="241" t="b">
+      <c r="B30" s="226" t="b">
         <v>0</v>
       </c>
       <c r="C30" s="163"/>
@@ -3876,34 +3884,55 @@
       <c r="N30" s="36"/>
       <c r="O30" s="36"/>
     </row>
-    <row r="31" spans="1:15" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="244" t="b">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="222" t="b">
         <v>0</v>
       </c>
-      <c r="B31" s="245" t="b">
-        <v>1</v>
-      </c>
-      <c r="C31" s="273"/>
-      <c r="D31" s="274">
-        <v>1</v>
-      </c>
-      <c r="E31" s="274" t="s">
+      <c r="B31" s="226" t="b">
+        <v>0</v>
+      </c>
+      <c r="C31" s="163"/>
+      <c r="D31" s="154"/>
+      <c r="E31" s="154"/>
+      <c r="F31" s="154"/>
+      <c r="G31" s="154"/>
+      <c r="H31" s="154"/>
+      <c r="I31" s="154"/>
+      <c r="J31" s="154"/>
+      <c r="K31" s="154"/>
+      <c r="L31" s="154"/>
+      <c r="M31" s="164"/>
+      <c r="N31" s="36"/>
+      <c r="O31" s="36"/>
+    </row>
+    <row r="32" spans="1:15" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="229" t="b">
+        <v>0</v>
+      </c>
+      <c r="B32" s="230" t="b">
+        <v>1</v>
+      </c>
+      <c r="C32" s="258"/>
+      <c r="D32" s="259">
+        <v>1</v>
+      </c>
+      <c r="E32" s="259" t="s">
         <v>119</v>
       </c>
-      <c r="F31" s="275"/>
-      <c r="G31" s="276" t="s">
+      <c r="F32" s="260"/>
+      <c r="G32" s="261" t="s">
         <v>166</v>
       </c>
-      <c r="H31" s="277"/>
-      <c r="I31" s="278" t="s">
+      <c r="H32" s="262"/>
+      <c r="I32" s="263" t="s">
         <v>208</v>
       </c>
-      <c r="J31" s="279"/>
-      <c r="K31" s="279"/>
-      <c r="L31" s="279"/>
-      <c r="M31" s="280"/>
-      <c r="N31" s="61"/>
-      <c r="O31" s="61"/>
+      <c r="J32" s="264"/>
+      <c r="K32" s="264"/>
+      <c r="L32" s="264"/>
+      <c r="M32" s="265"/>
+      <c r="N32" s="61"/>
+      <c r="O32" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3911,7 +3940,7 @@
     <mergeCell ref="E3:M4"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <conditionalFormatting sqref="A6:B31">
+  <conditionalFormatting sqref="A6:B32">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -3950,17 +3979,17 @@
       <c r="B1" s="40">
         <v>1</v>
       </c>
-      <c r="C1" s="228" t="s">
+      <c r="C1" s="266" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="229"/>
-      <c r="E1" s="229"/>
-      <c r="F1" s="229"/>
-      <c r="G1" s="229"/>
-      <c r="H1" s="229"/>
-      <c r="I1" s="229"/>
-      <c r="J1" s="229"/>
-      <c r="K1" s="230"/>
+      <c r="D1" s="267"/>
+      <c r="E1" s="267"/>
+      <c r="F1" s="267"/>
+      <c r="G1" s="267"/>
+      <c r="H1" s="267"/>
+      <c r="I1" s="267"/>
+      <c r="J1" s="267"/>
+      <c r="K1" s="268"/>
       <c r="L1" s="36"/>
       <c r="M1" s="36"/>
     </row>
@@ -3971,15 +4000,15 @@
       <c r="B2" s="40">
         <v>1</v>
       </c>
-      <c r="C2" s="231"/>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
-      <c r="G2" s="232"/>
-      <c r="H2" s="232"/>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="233"/>
+      <c r="C2" s="269"/>
+      <c r="D2" s="270"/>
+      <c r="E2" s="270"/>
+      <c r="F2" s="270"/>
+      <c r="G2" s="270"/>
+      <c r="H2" s="270"/>
+      <c r="I2" s="270"/>
+      <c r="J2" s="270"/>
+      <c r="K2" s="271"/>
       <c r="L2" s="36"/>
       <c r="M2" s="36"/>
     </row>
@@ -3990,17 +4019,17 @@
       <c r="B3" s="40">
         <v>1</v>
       </c>
-      <c r="C3" s="222" t="s">
+      <c r="C3" s="272" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="223"/>
-      <c r="E3" s="223"/>
-      <c r="F3" s="223"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="223"/>
-      <c r="I3" s="223"/>
-      <c r="J3" s="223"/>
-      <c r="K3" s="224"/>
+      <c r="D3" s="273"/>
+      <c r="E3" s="273"/>
+      <c r="F3" s="273"/>
+      <c r="G3" s="273"/>
+      <c r="H3" s="273"/>
+      <c r="I3" s="273"/>
+      <c r="J3" s="273"/>
+      <c r="K3" s="274"/>
       <c r="L3" s="36"/>
       <c r="M3" s="36"/>
     </row>
@@ -4011,15 +4040,15 @@
       <c r="B4" s="132">
         <v>46017</v>
       </c>
-      <c r="C4" s="225"/>
-      <c r="D4" s="226"/>
-      <c r="E4" s="226"/>
-      <c r="F4" s="226"/>
-      <c r="G4" s="226"/>
-      <c r="H4" s="226"/>
-      <c r="I4" s="226"/>
-      <c r="J4" s="226"/>
-      <c r="K4" s="227"/>
+      <c r="C4" s="275"/>
+      <c r="D4" s="276"/>
+      <c r="E4" s="276"/>
+      <c r="F4" s="276"/>
+      <c r="G4" s="276"/>
+      <c r="H4" s="276"/>
+      <c r="I4" s="276"/>
+      <c r="J4" s="276"/>
+      <c r="K4" s="277"/>
       <c r="L4" s="36"/>
       <c r="M4" s="36"/>
     </row>
@@ -4061,7 +4090,7 @@
       <c r="M5" s="108"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="246" t="s">
+      <c r="A6" s="231" t="s">
         <v>92</v>
       </c>
       <c r="B6" s="134">
@@ -4090,7 +4119,7 @@
       <c r="M6" s="36"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="247"/>
+      <c r="A7" s="232"/>
       <c r="B7" s="85">
         <v>1</v>
       </c>
@@ -4117,7 +4146,7 @@
       <c r="M7" s="36"/>
     </row>
     <row r="8" spans="1:13" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="248"/>
+      <c r="A8" s="233"/>
       <c r="B8" s="101">
         <v>1</v>
       </c>
@@ -4144,7 +4173,7 @@
       <c r="M8" s="108"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="249" t="s">
+      <c r="A9" s="234" t="s">
         <v>100</v>
       </c>
       <c r="B9" s="93">
@@ -4171,7 +4200,7 @@
       <c r="M9" s="36"/>
     </row>
     <row r="10" spans="1:13" s="60" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="250"/>
+      <c r="A10" s="235"/>
       <c r="B10" s="62">
         <v>2</v>
       </c>
@@ -4196,7 +4225,7 @@
       <c r="M10" s="61"/>
     </row>
     <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="251"/>
+      <c r="A11" s="236"/>
       <c r="B11" s="62">
         <v>1</v>
       </c>
@@ -4221,7 +4250,7 @@
       <c r="K11" s="80"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="252"/>
+      <c r="A12" s="237"/>
       <c r="B12" s="110">
         <v>2</v>
       </c>
@@ -4246,7 +4275,7 @@
       <c r="M12" s="36"/>
     </row>
     <row r="13" spans="1:13" s="182" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="253"/>
+      <c r="A13" s="238"/>
       <c r="B13" s="125">
         <v>1</v>
       </c>
@@ -4271,7 +4300,7 @@
       <c r="M13" s="181"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="254" t="s">
+      <c r="A14" s="239" t="s">
         <v>225</v>
       </c>
       <c r="B14" s="173">
@@ -4300,7 +4329,7 @@
       <c r="M14" s="36"/>
     </row>
     <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="255"/>
+      <c r="A15" s="240"/>
       <c r="B15" s="146">
         <v>12</v>
       </c>
@@ -4327,7 +4356,7 @@
       <c r="M15" s="36"/>
     </row>
     <row r="16" spans="1:13" s="194" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="255"/>
+      <c r="A16" s="240"/>
       <c r="B16" s="146">
         <v>1</v>
       </c>
@@ -4354,7 +4383,7 @@
       <c r="M16" s="193"/>
     </row>
     <row r="17" spans="1:13" s="192" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="256"/>
+      <c r="A17" s="241"/>
       <c r="B17" s="184">
         <v>2</v>
       </c>
@@ -4381,7 +4410,7 @@
       <c r="M17" s="191"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="257" t="s">
+      <c r="A18" s="242" t="s">
         <v>185</v>
       </c>
       <c r="B18" s="117">
@@ -4410,7 +4439,7 @@
       <c r="M18" s="36"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="258"/>
+      <c r="A19" s="243"/>
       <c r="B19" s="69">
         <v>1</v>
       </c>
@@ -4437,7 +4466,7 @@
       <c r="M19" s="36"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="258"/>
+      <c r="A20" s="243"/>
       <c r="B20" s="69">
         <v>1</v>
       </c>
@@ -4464,7 +4493,7 @@
       <c r="M20" s="36"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="258"/>
+      <c r="A21" s="243"/>
       <c r="B21" s="75">
         <v>2</v>
       </c>
@@ -4491,7 +4520,7 @@
       <c r="M21" s="36"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="258"/>
+      <c r="A22" s="243"/>
       <c r="B22" s="75">
         <v>1</v>
       </c>
@@ -4518,7 +4547,7 @@
       <c r="M22" s="36"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="258"/>
+      <c r="A23" s="243"/>
       <c r="B23" s="75">
         <v>1</v>
       </c>
@@ -4545,7 +4574,7 @@
       <c r="M23" s="36"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="258"/>
+      <c r="A24" s="243"/>
       <c r="B24" s="75">
         <v>2</v>
       </c>
@@ -4572,7 +4601,7 @@
       <c r="M24" s="36"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="258"/>
+      <c r="A25" s="243"/>
       <c r="B25" s="75">
         <v>2</v>
       </c>
@@ -4599,7 +4628,7 @@
       <c r="M25" s="36"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="259"/>
+      <c r="A26" s="244"/>
       <c r="B26" s="196">
         <v>2</v>
       </c>
@@ -4626,7 +4655,7 @@
       <c r="M26" s="36"/>
     </row>
     <row r="27" spans="1:13" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="260"/>
+      <c r="A27" s="245"/>
       <c r="B27" s="213">
         <v>1</v>
       </c>
@@ -4653,7 +4682,7 @@
       <c r="M27" s="108"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="261" t="s">
+      <c r="A28" s="246" t="s">
         <v>226</v>
       </c>
       <c r="B28" s="205">
@@ -4680,8 +4709,8 @@
       <c r="M28" s="36"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="262"/>
-      <c r="B29" s="263"/>
+      <c r="A29" s="247"/>
+      <c r="B29" s="248"/>
       <c r="C29" s="155"/>
       <c r="D29" s="156"/>
       <c r="E29" s="154"/>
@@ -4695,8 +4724,8 @@
       <c r="M29" s="36"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="262"/>
-      <c r="B30" s="263"/>
+      <c r="A30" s="247"/>
+      <c r="B30" s="248"/>
       <c r="C30" s="154"/>
       <c r="D30" s="154"/>
       <c r="E30" s="154"/>
@@ -4710,8 +4739,8 @@
       <c r="M30" s="36"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="262"/>
-      <c r="B31" s="263"/>
+      <c r="A31" s="247"/>
+      <c r="B31" s="248"/>
       <c r="C31" s="154"/>
       <c r="D31" s="154"/>
       <c r="E31" s="154"/>
@@ -4725,7 +4754,7 @@
       <c r="M31" s="36"/>
     </row>
     <row r="32" spans="1:13" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="264"/>
+      <c r="A32" s="249"/>
       <c r="B32" s="165">
         <v>1</v>
       </c>
@@ -4779,14 +4808,14 @@
       <c r="E2" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="234" t="s">
+      <c r="F2" s="278" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="234"/>
-      <c r="H2" s="234"/>
-      <c r="I2" s="234"/>
-      <c r="J2" s="234"/>
-      <c r="K2" s="234"/>
+      <c r="G2" s="278"/>
+      <c r="H2" s="278"/>
+      <c r="I2" s="278"/>
+      <c r="J2" s="278"/>
+      <c r="K2" s="278"/>
       <c r="L2" s="59" t="s">
         <v>149</v>
       </c>

</xml_diff>

<commit_message>
remaining files i forgor
</commit_message>
<xml_diff>
--- a/Documents/OMNIXIE_sheets.xlsx
+++ b/Documents/OMNIXIE_sheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21nic\OneDrive\Desktop\NIXIE\OMNIXIE\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADE8EB2-ADF0-49D9-87D9-7E859E73AA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA67E55-8EE9-466C-BFD4-3BCE711FE6AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="247">
   <si>
     <t>A: ADC, A7 (ADC_IN7)</t>
   </si>
@@ -769,6 +769,18 @@
   </si>
   <si>
     <t>R10,R16</t>
+  </si>
+  <si>
+    <t>RK0971114D0B</t>
+  </si>
+  <si>
+    <t>potentiometer</t>
+  </si>
+  <si>
+    <t>BM03B-SRSS-TB</t>
+  </si>
+  <si>
+    <t>For Later Use</t>
   </si>
 </sst>
 </file>
@@ -1643,7 +1655,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="279">
+  <cellXfs count="290">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2282,7 +2294,6 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2298,8 +2309,6 @@
     <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2369,6 +2378,46 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2924,7 +2973,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE706952-430C-44AA-84E6-C88695E38A9F}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
@@ -2951,17 +3000,17 @@
       <c r="D1" s="40">
         <v>1</v>
       </c>
-      <c r="E1" s="266" t="s">
+      <c r="E1" s="263" t="s">
         <v>139</v>
       </c>
-      <c r="F1" s="267"/>
-      <c r="G1" s="267"/>
-      <c r="H1" s="267"/>
-      <c r="I1" s="267"/>
-      <c r="J1" s="267"/>
-      <c r="K1" s="267"/>
-      <c r="L1" s="267"/>
-      <c r="M1" s="268"/>
+      <c r="F1" s="264"/>
+      <c r="G1" s="264"/>
+      <c r="H1" s="264"/>
+      <c r="I1" s="264"/>
+      <c r="J1" s="264"/>
+      <c r="K1" s="264"/>
+      <c r="L1" s="264"/>
+      <c r="M1" s="265"/>
       <c r="N1" s="36"/>
       <c r="O1" s="36"/>
     </row>
@@ -2974,15 +3023,15 @@
       <c r="D2" s="40">
         <v>1</v>
       </c>
-      <c r="E2" s="269"/>
-      <c r="F2" s="270"/>
-      <c r="G2" s="270"/>
-      <c r="H2" s="270"/>
-      <c r="I2" s="270"/>
-      <c r="J2" s="270"/>
-      <c r="K2" s="270"/>
-      <c r="L2" s="270"/>
-      <c r="M2" s="271"/>
+      <c r="E2" s="266"/>
+      <c r="F2" s="267"/>
+      <c r="G2" s="267"/>
+      <c r="H2" s="267"/>
+      <c r="I2" s="267"/>
+      <c r="J2" s="267"/>
+      <c r="K2" s="267"/>
+      <c r="L2" s="267"/>
+      <c r="M2" s="268"/>
       <c r="N2" s="36"/>
       <c r="O2" s="36"/>
     </row>
@@ -2995,17 +3044,17 @@
       <c r="D3" s="40">
         <v>1</v>
       </c>
-      <c r="E3" s="272" t="s">
+      <c r="E3" s="269" t="s">
         <v>141</v>
       </c>
-      <c r="F3" s="273"/>
-      <c r="G3" s="273"/>
-      <c r="H3" s="273"/>
-      <c r="I3" s="273"/>
-      <c r="J3" s="273"/>
-      <c r="K3" s="273"/>
-      <c r="L3" s="273"/>
-      <c r="M3" s="274"/>
+      <c r="F3" s="270"/>
+      <c r="G3" s="270"/>
+      <c r="H3" s="270"/>
+      <c r="I3" s="270"/>
+      <c r="J3" s="270"/>
+      <c r="K3" s="270"/>
+      <c r="L3" s="270"/>
+      <c r="M3" s="271"/>
       <c r="N3" s="36"/>
       <c r="O3" s="36"/>
     </row>
@@ -3018,15 +3067,15 @@
       <c r="D4" s="132">
         <v>46017</v>
       </c>
-      <c r="E4" s="275"/>
-      <c r="F4" s="276"/>
-      <c r="G4" s="276"/>
-      <c r="H4" s="276"/>
-      <c r="I4" s="276"/>
-      <c r="J4" s="276"/>
-      <c r="K4" s="276"/>
-      <c r="L4" s="276"/>
-      <c r="M4" s="277"/>
+      <c r="E4" s="272"/>
+      <c r="F4" s="273"/>
+      <c r="G4" s="273"/>
+      <c r="H4" s="273"/>
+      <c r="I4" s="273"/>
+      <c r="J4" s="273"/>
+      <c r="K4" s="273"/>
+      <c r="L4" s="273"/>
+      <c r="M4" s="274"/>
       <c r="N4" s="36"/>
       <c r="O4" s="36"/>
     </row>
@@ -3075,7 +3124,7 @@
     </row>
     <row r="6" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="222" t="b">
         <v>1</v>
@@ -3110,7 +3159,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" s="223" t="b">
         <v>1</v>
@@ -3143,7 +3192,7 @@
     </row>
     <row r="8" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" s="224" t="b">
         <v>1</v>
@@ -3176,7 +3225,7 @@
     </row>
     <row r="9" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" s="222" t="b">
         <v>1</v>
@@ -3240,7 +3289,7 @@
     </row>
     <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" s="226" t="b">
         <v>1</v>
@@ -3271,7 +3320,7 @@
     </row>
     <row r="12" spans="1:15" s="182" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" s="224" t="b">
         <v>1</v>
@@ -3302,7 +3351,7 @@
     </row>
     <row r="13" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A13" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" s="222" t="b">
         <v>1</v>
@@ -3337,7 +3386,7 @@
     </row>
     <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" s="226" t="b">
         <v>1</v>
@@ -3370,7 +3419,7 @@
     </row>
     <row r="15" spans="1:15" s="194" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" s="226" t="b">
         <v>1</v>
@@ -3403,7 +3452,7 @@
     </row>
     <row r="16" spans="1:15" s="192" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" s="227" t="b">
         <v>1</v>
@@ -3471,7 +3520,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" s="226" t="b">
         <v>1</v>
@@ -3537,7 +3586,7 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" s="226" t="b">
         <v>1</v>
@@ -3603,7 +3652,7 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" s="226" t="b">
         <v>1</v>
@@ -3800,8 +3849,8 @@
       <c r="O27" s="108"/>
     </row>
     <row r="28" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="222" t="b">
-        <v>0</v>
+      <c r="A28" s="228" t="b">
+        <v>1</v>
       </c>
       <c r="B28" s="228" t="b">
         <v>1</v>
@@ -3809,7 +3858,7 @@
       <c r="C28" s="204" t="s">
         <v>226</v>
       </c>
-      <c r="D28" s="205">
+      <c r="D28" s="207">
         <v>1</v>
       </c>
       <c r="E28" s="205" t="s">
@@ -3832,72 +3881,78 @@
       <c r="N28" s="36"/>
       <c r="O28" s="36"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="222" t="b">
+    <row r="29" spans="1:15" s="109" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="281" t="b">
         <v>0</v>
       </c>
-      <c r="B29" s="223" t="b">
-        <v>1</v>
-      </c>
-      <c r="C29" s="250"/>
-      <c r="D29" s="251">
+      <c r="B29" s="224" t="b">
+        <v>0</v>
+      </c>
+      <c r="C29" s="282"/>
+      <c r="D29" s="283"/>
+      <c r="E29" s="284"/>
+      <c r="F29" s="285"/>
+      <c r="G29" s="283"/>
+      <c r="H29" s="286"/>
+      <c r="I29" s="287"/>
+      <c r="J29" s="288"/>
+      <c r="K29" s="288"/>
+      <c r="L29" s="288"/>
+      <c r="M29" s="289"/>
+      <c r="N29" s="108"/>
+      <c r="O29" s="108"/>
+    </row>
+    <row r="30" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="222" t="b">
+        <v>1</v>
+      </c>
+      <c r="B30" s="276" t="b">
+        <v>1</v>
+      </c>
+      <c r="C30" s="277" t="s">
+        <v>246</v>
+      </c>
+      <c r="D30" s="278">
         <v>2</v>
       </c>
-      <c r="E29" s="251" t="s">
-        <v>101</v>
-      </c>
-      <c r="F29" s="252" t="s">
-        <v>190</v>
-      </c>
-      <c r="G29" s="253" t="s">
-        <v>166</v>
-      </c>
-      <c r="H29" s="254"/>
-      <c r="I29" s="255" t="s">
-        <v>102</v>
-      </c>
-      <c r="J29" s="256"/>
-      <c r="K29" s="256"/>
-      <c r="L29" s="256"/>
-      <c r="M29" s="257"/>
-      <c r="N29" s="36"/>
-      <c r="O29" s="36"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="222" t="b">
-        <v>0</v>
-      </c>
-      <c r="B30" s="226" t="b">
-        <v>0</v>
-      </c>
-      <c r="C30" s="163"/>
-      <c r="D30" s="154"/>
-      <c r="E30" s="154"/>
-      <c r="F30" s="154"/>
-      <c r="G30" s="154"/>
-      <c r="H30" s="154"/>
-      <c r="I30" s="154"/>
-      <c r="J30" s="154"/>
-      <c r="K30" s="154"/>
-      <c r="L30" s="154"/>
-      <c r="M30" s="164"/>
+      <c r="E30" s="205" t="s">
+        <v>245</v>
+      </c>
+      <c r="F30" s="279"/>
+      <c r="G30" s="279"/>
+      <c r="H30" s="279"/>
+      <c r="I30" s="279"/>
+      <c r="J30" s="279"/>
+      <c r="K30" s="279"/>
+      <c r="L30" s="279"/>
+      <c r="M30" s="280"/>
       <c r="N30" s="36"/>
       <c r="O30" s="36"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B31" s="226" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" s="163"/>
-      <c r="D31" s="154"/>
-      <c r="E31" s="154"/>
-      <c r="F31" s="154"/>
-      <c r="G31" s="154"/>
-      <c r="H31" s="154"/>
-      <c r="I31" s="154"/>
+      <c r="D31" s="252">
+        <v>2</v>
+      </c>
+      <c r="E31" s="250" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="251" t="s">
+        <v>190</v>
+      </c>
+      <c r="G31" s="252" t="s">
+        <v>166</v>
+      </c>
+      <c r="H31" s="253"/>
+      <c r="I31" s="254" t="s">
+        <v>102</v>
+      </c>
       <c r="J31" s="154"/>
       <c r="K31" s="154"/>
       <c r="L31" s="154"/>
@@ -3907,32 +3962,40 @@
     </row>
     <row r="32" spans="1:15" s="60" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="229" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B32" s="230" t="b">
         <v>1</v>
       </c>
-      <c r="C32" s="258"/>
-      <c r="D32" s="259">
-        <v>1</v>
-      </c>
-      <c r="E32" s="259" t="s">
+      <c r="C32" s="255"/>
+      <c r="D32" s="256">
+        <v>1</v>
+      </c>
+      <c r="E32" s="256" t="s">
         <v>119</v>
       </c>
-      <c r="F32" s="260"/>
-      <c r="G32" s="261" t="s">
+      <c r="F32" s="257"/>
+      <c r="G32" s="258" t="s">
         <v>166</v>
       </c>
-      <c r="H32" s="262"/>
-      <c r="I32" s="263" t="s">
+      <c r="H32" s="259"/>
+      <c r="I32" s="260" t="s">
         <v>208</v>
       </c>
-      <c r="J32" s="264"/>
-      <c r="K32" s="264"/>
-      <c r="L32" s="264"/>
-      <c r="M32" s="265"/>
+      <c r="J32" s="261"/>
+      <c r="K32" s="261"/>
+      <c r="L32" s="261"/>
+      <c r="M32" s="262"/>
       <c r="N32" s="61"/>
       <c r="O32" s="61"/>
+    </row>
+    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
+        <v>243</v>
+      </c>
+      <c r="F36" t="s">
+        <v>244</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3979,17 +4042,17 @@
       <c r="B1" s="40">
         <v>1</v>
       </c>
-      <c r="C1" s="266" t="s">
+      <c r="C1" s="263" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="267"/>
-      <c r="E1" s="267"/>
-      <c r="F1" s="267"/>
-      <c r="G1" s="267"/>
-      <c r="H1" s="267"/>
-      <c r="I1" s="267"/>
-      <c r="J1" s="267"/>
-      <c r="K1" s="268"/>
+      <c r="D1" s="264"/>
+      <c r="E1" s="264"/>
+      <c r="F1" s="264"/>
+      <c r="G1" s="264"/>
+      <c r="H1" s="264"/>
+      <c r="I1" s="264"/>
+      <c r="J1" s="264"/>
+      <c r="K1" s="265"/>
       <c r="L1" s="36"/>
       <c r="M1" s="36"/>
     </row>
@@ -4000,15 +4063,15 @@
       <c r="B2" s="40">
         <v>1</v>
       </c>
-      <c r="C2" s="269"/>
-      <c r="D2" s="270"/>
-      <c r="E2" s="270"/>
-      <c r="F2" s="270"/>
-      <c r="G2" s="270"/>
-      <c r="H2" s="270"/>
-      <c r="I2" s="270"/>
-      <c r="J2" s="270"/>
-      <c r="K2" s="271"/>
+      <c r="C2" s="266"/>
+      <c r="D2" s="267"/>
+      <c r="E2" s="267"/>
+      <c r="F2" s="267"/>
+      <c r="G2" s="267"/>
+      <c r="H2" s="267"/>
+      <c r="I2" s="267"/>
+      <c r="J2" s="267"/>
+      <c r="K2" s="268"/>
       <c r="L2" s="36"/>
       <c r="M2" s="36"/>
     </row>
@@ -4019,17 +4082,17 @@
       <c r="B3" s="40">
         <v>1</v>
       </c>
-      <c r="C3" s="272" t="s">
+      <c r="C3" s="269" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="273"/>
-      <c r="E3" s="273"/>
-      <c r="F3" s="273"/>
-      <c r="G3" s="273"/>
-      <c r="H3" s="273"/>
-      <c r="I3" s="273"/>
-      <c r="J3" s="273"/>
-      <c r="K3" s="274"/>
+      <c r="D3" s="270"/>
+      <c r="E3" s="270"/>
+      <c r="F3" s="270"/>
+      <c r="G3" s="270"/>
+      <c r="H3" s="270"/>
+      <c r="I3" s="270"/>
+      <c r="J3" s="270"/>
+      <c r="K3" s="271"/>
       <c r="L3" s="36"/>
       <c r="M3" s="36"/>
     </row>
@@ -4040,15 +4103,15 @@
       <c r="B4" s="132">
         <v>46017</v>
       </c>
-      <c r="C4" s="275"/>
-      <c r="D4" s="276"/>
-      <c r="E4" s="276"/>
-      <c r="F4" s="276"/>
-      <c r="G4" s="276"/>
-      <c r="H4" s="276"/>
-      <c r="I4" s="276"/>
-      <c r="J4" s="276"/>
-      <c r="K4" s="277"/>
+      <c r="C4" s="272"/>
+      <c r="D4" s="273"/>
+      <c r="E4" s="273"/>
+      <c r="F4" s="273"/>
+      <c r="G4" s="273"/>
+      <c r="H4" s="273"/>
+      <c r="I4" s="273"/>
+      <c r="J4" s="273"/>
+      <c r="K4" s="274"/>
       <c r="L4" s="36"/>
       <c r="M4" s="36"/>
     </row>
@@ -4808,14 +4871,14 @@
       <c r="E2" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="278" t="s">
+      <c r="F2" s="275" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="278"/>
-      <c r="H2" s="278"/>
-      <c r="I2" s="278"/>
-      <c r="J2" s="278"/>
-      <c r="K2" s="278"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
       <c r="L2" s="59" t="s">
         <v>149</v>
       </c>

</xml_diff>